<commit_message>
Add new mission ROI samples and refresh workbook
</commit_message>
<xml_diff>
--- a/downloads/orion-mission-research.xlsx
+++ b/downloads/orion-mission-research.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Reca6cfc8997c43b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mission Data" sheetId="2" r:id="R6c6287ba5281467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="Ra0bb18af9ddc4567"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R99703f4a7d794c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mission Data" sheetId="2" r:id="R2a4dd6de806d40df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R9ef7e876788b4862"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -195,8 +195,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MissionSamples" displayName="MissionSamples" ref="A1:AA66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:AA66"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MissionSamples" displayName="MissionSamples" ref="A1:AA101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:AA101"/>
   <x:tableColumns count="27">
     <x:tableColumn id="1" name="Record ID"/>
     <x:tableColumn id="2" name="Observed date"/>
@@ -497,15 +497,15 @@
       </x:c>
       <x:c r="B5" s="14" t="n">
         <x:f>COUNTIF('Mission Data'!$C$2:$C$1000,A5)</x:f>
-        <x:v>24</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C5" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A5,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>23</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D5" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A5,'Mission Data'!$Z$2:$Z$1000,"Yes",'Mission Data'!$X$2:$X$1000,"&gt;0")</x:f>
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E5" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A5,'Mission Data'!$Z$2:$Z$1000,"Yes",'Mission Data'!$X$2:$X$1000,"&lt;0")</x:f>
@@ -517,7 +517,7 @@
       </x:c>
       <x:c r="G5" s="28" t="n">
         <x:f>_xlfn.MAXIFS('Mission Data'!$Y$2:$Y$1000,'Mission Data'!$C$2:$C$1000,A5,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>3.569279444006227</x:v>
+        <x:v>5.649927762383938</x:v>
       </x:c>
       <x:c r="H5" s="29" t="n">
         <x:f>_xlfn.MINIFS('Mission Data'!$X$2:$X$1000,'Mission Data'!$C$2:$C$1000,A5,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
@@ -525,7 +525,7 @@
       </x:c>
       <x:c r="I5" s="29" t="n">
         <x:f>_xlfn.MAXIFS('Mission Data'!$X$2:$X$1000,'Mission Data'!$C$2:$C$1000,A5,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>53718117</x:v>
+        <x:v>299113884</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -534,35 +534,35 @@
       </x:c>
       <x:c r="B6" s="14" t="n">
         <x:f>COUNTIF('Mission Data'!$C$2:$C$1000,A6)</x:f>
-        <x:v>20</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C6" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A6,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>15</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D6" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A6,'Mission Data'!$Z$2:$Z$1000,"Yes",'Mission Data'!$X$2:$X$1000,"&gt;0")</x:f>
-        <x:v>14</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E6" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A6,'Mission Data'!$Z$2:$Z$1000,"Yes",'Mission Data'!$X$2:$X$1000,"&lt;0")</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="28" t="n">
         <x:f>_xlfn.MINIFS('Mission Data'!$Y$2:$Y$1000,'Mission Data'!$C$2:$C$1000,A6,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>0.6596787413878826</x:v>
+        <x:v>0.46209403984884917</x:v>
       </x:c>
       <x:c r="G6" s="28" t="n">
         <x:f>_xlfn.MAXIFS('Mission Data'!$Y$2:$Y$1000,'Mission Data'!$C$2:$C$1000,A6,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>5.728507043673295</x:v>
+        <x:v>8.621369147490276</x:v>
       </x:c>
       <x:c r="H6" s="29" t="n">
         <x:f>_xlfn.MINIFS('Mission Data'!$X$2:$X$1000,'Mission Data'!$C$2:$C$1000,A6,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>-14374149</x:v>
+        <x:v>-18790131</x:v>
       </x:c>
       <x:c r="I6" s="29" t="n">
         <x:f>_xlfn.MAXIFS('Mission Data'!$X$2:$X$1000,'Mission Data'!$C$2:$C$1000,A6,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>187631888</x:v>
+        <x:v>487851460.5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -571,15 +571,15 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>COUNTIF('Mission Data'!$C$2:$C$1000,A7)</x:f>
-        <x:v>20</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C7" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A7,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>19</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D7" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A7,'Mission Data'!$Z$2:$Z$1000,"Yes",'Mission Data'!$X$2:$X$1000,"&gt;0")</x:f>
-        <x:v>16</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E7" s="14" t="n">
         <x:f>COUNTIFS('Mission Data'!$C$2:$C$1000,A7,'Mission Data'!$Z$2:$Z$1000,"Yes",'Mission Data'!$X$2:$X$1000,"&lt;0")</x:f>
@@ -591,7 +591,7 @@
       </x:c>
       <x:c r="G7" s="28" t="n">
         <x:f>_xlfn.MAXIFS('Mission Data'!$Y$2:$Y$1000,'Mission Data'!$C$2:$C$1000,A7,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>6.052134289439374</x:v>
+        <x:v>9.295034466964388</x:v>
       </x:c>
       <x:c r="H7" s="29" t="n">
         <x:f>_xlfn.MINIFS('Mission Data'!$X$2:$X$1000,'Mission Data'!$C$2:$C$1000,A7,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
@@ -599,7 +599,7 @@
       </x:c>
       <x:c r="I7" s="29" t="n">
         <x:f>_xlfn.MAXIFS('Mission Data'!$X$2:$X$1000,'Mission Data'!$C$2:$C$1000,A7,'Mission Data'!$Z$2:$Z$1000,"Yes")</x:f>
-        <x:v>63155731.5</x:v>
+        <x:v>234327508.5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -616,7 +616,7 @@
       </x:c>
       <x:c r="B10" s="14" t="n">
         <x:f>COUNTA('Mission Data'!$A$2:$A$1000)</x:f>
-        <x:v>65</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -625,7 +625,7 @@
       </x:c>
       <x:c r="B11" s="14" t="n">
         <x:f>COUNTIF('Mission Data'!$M$2:$M$1000,"possible")</x:f>
-        <x:v>64</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -6527,28 +6527,28 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="20" t="str">
-        <x:v>delivery-metal-626-pve-4star-collected</x:v>
+        <x:v>s10-20261002-01</x:v>
       </x:c>
       <x:c r="B66" s="21" t="n">
-        <x:v>46296</x:v>
-      </x:c>
-      <x:c r="C66" s="22" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C66" s="22" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D66" s="20" t="str">
-        <x:v>PTS reward claim dialog</x:v>
+        <x:v>PTS scan card</x:v>
       </x:c>
       <x:c r="E66" s="20" t="str">
         <x:v>Delivery: Metal</x:v>
       </x:c>
       <x:c r="F66" s="20" t="str">
-        <x:v>PvE</x:v>
+        <x:v>PvP</x:v>
       </x:c>
       <x:c r="G66" s="23" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H66" s="23" t="n">
-        <x:v>626</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="I66" s="23" t="str">
         <x:v>Delivery</x:v>
@@ -6557,16 +6557,16 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="K66" s="23" t="n">
-        <x:v>90</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="L66" s="23" t="n">
         <x:v>3555</x:v>
       </x:c>
       <x:c r="M66" s="20" t="str">
-        <x:v>collected</x:v>
+        <x:v>possible</x:v>
       </x:c>
       <x:c r="N66" s="23" t="n">
-        <x:v>59634076</x:v>
+        <x:v>363442884</x:v>
       </x:c>
       <x:c r="O66" s="23" t="n">
         <x:v>0</x:v>
@@ -6578,32 +6578,32 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="R66" s="24" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S66" s="23" t="n">
-        <x:v>14073696</x:v>
+        <x:v>21443000</x:v>
       </x:c>
       <x:c r="T66" s="24" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U66" s="24" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="V66" s="25" t="n">
         <x:f>N66+1.5*O66+3*P66+3*Q66</x:f>
-        <x:v>59634076</x:v>
+        <x:v>363442884</x:v>
       </x:c>
       <x:c r="W66" s="25" t="n">
         <x:f>S66*3</x:f>
-        <x:v>42221088</x:v>
+        <x:v>64329000</x:v>
       </x:c>
       <x:c r="X66" s="25" t="n">
         <x:f>IF(Z66="No",0,V66-W66)</x:f>
-        <x:v>17412988</x:v>
+        <x:v>299113884</x:v>
       </x:c>
       <x:c r="Y66" s="26" t="n">
         <x:f>IF(Z66="No",0,IFERROR(V66/W66,0))</x:f>
-        <x:v>1.4124239526939713</x:v>
+        <x:v>5.649751807116542</x:v>
       </x:c>
       <x:c r="Z66" s="27" t="str">
         <x:f>IF(AND(U66=TRUE,V66=0),"No","Yes")</x:f>
@@ -6614,15 +6614,3130 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="20" t="str">
+        <x:v>s10-20261002-02</x:v>
+      </x:c>
+      <x:c r="B67" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C67" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D67" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E67" s="20" t="str">
+        <x:v>Small Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F67" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G67" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H67" s="23" t="n">
+        <x:v>594</x:v>
+      </x:c>
+      <x:c r="I67" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J67" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K67" s="23" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="L67" s="23" t="n">
+        <x:v>3270</x:v>
+      </x:c>
+      <x:c r="M67" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N67" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O67" s="23" t="n">
+        <x:v>116561398</x:v>
+      </x:c>
+      <x:c r="P67" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q67" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R67" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S67" s="23" t="n">
+        <x:v>16878000</x:v>
+      </x:c>
+      <x:c r="T67" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U67" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V67" s="25" t="n">
+        <x:f>N67+1.5*O67+3*P67+3*Q67</x:f>
+        <x:v>174842097</x:v>
+      </x:c>
+      <x:c r="W67" s="25" t="n">
+        <x:f>S67*3</x:f>
+        <x:v>50634000</x:v>
+      </x:c>
+      <x:c r="X67" s="25" t="n">
+        <x:f>IF(Z67="No",0,V67-W67)</x:f>
+        <x:v>124208097</x:v>
+      </x:c>
+      <x:c r="Y67" s="26" t="n">
+        <x:f>IF(Z67="No",0,IFERROR(V67/W67,0))</x:f>
+        <x:v>3.453057175020737</x:v>
+      </x:c>
+      <x:c r="Z67" s="27" t="str">
+        <x:f>IF(AND(U67=TRUE,V67=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA67" s="27" t="str">
+        <x:f>IF(Z67="No","Not comparable",IF(X67&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="20" t="str">
+        <x:v>s10-20261002-03</x:v>
+      </x:c>
+      <x:c r="B68" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C68" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D68" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E68" s="20" t="str">
+        <x:v>Rescue</x:v>
+      </x:c>
+      <x:c r="F68" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G68" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H68" s="23" t="n">
+        <x:v>732</x:v>
+      </x:c>
+      <x:c r="I68" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J68" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K68" s="23" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="L68" s="23" t="n">
+        <x:v>3270</x:v>
+      </x:c>
+      <x:c r="M68" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N68" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O68" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P68" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q68" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R68" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S68" s="23" t="n">
+        <x:v>5546000</x:v>
+      </x:c>
+      <x:c r="T68" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U68" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V68" s="25" t="n">
+        <x:f>N68+1.5*O68+3*P68+3*Q68</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W68" s="25" t="n">
+        <x:f>S68*3</x:f>
+        <x:v>16638000</x:v>
+      </x:c>
+      <x:c r="X68" s="25" t="n">
+        <x:f>IF(Z68="No",0,V68-W68)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y68" s="26" t="n">
+        <x:f>IF(Z68="No",0,IFERROR(V68/W68,0))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z68" s="27" t="str">
+        <x:f>IF(AND(U68=TRUE,V68=0),"No","Yes")</x:f>
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AA68" s="27" t="str">
+        <x:f>IF(Z68="No","Not comparable",IF(X68&gt;0,"Yes","No"))</x:f>
+        <x:v>Not comparable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="20" t="str">
+        <x:v>s10-20261002-04</x:v>
+      </x:c>
+      <x:c r="B69" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C69" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D69" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E69" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F69" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G69" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H69" s="23" t="n">
+        <x:v>543</x:v>
+      </x:c>
+      <x:c r="I69" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J69" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K69" s="23" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="L69" s="23" t="n">
+        <x:v>2985</x:v>
+      </x:c>
+      <x:c r="M69" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N69" s="23" t="n">
+        <x:v>348673992</x:v>
+      </x:c>
+      <x:c r="O69" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P69" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q69" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R69" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S69" s="23" t="n">
+        <x:v>20571000</x:v>
+      </x:c>
+      <x:c r="T69" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U69" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V69" s="25" t="n">
+        <x:f>N69+1.5*O69+3*P69+3*Q69</x:f>
+        <x:v>348673992</x:v>
+      </x:c>
+      <x:c r="W69" s="25" t="n">
+        <x:f>S69*3</x:f>
+        <x:v>61713000</x:v>
+      </x:c>
+      <x:c r="X69" s="25" t="n">
+        <x:f>IF(Z69="No",0,V69-W69)</x:f>
+        <x:v>286960992</x:v>
+      </x:c>
+      <x:c r="Y69" s="26" t="n">
+        <x:f>IF(Z69="No",0,IFERROR(V69/W69,0))</x:f>
+        <x:v>5.649927762383938</x:v>
+      </x:c>
+      <x:c r="Z69" s="27" t="str">
+        <x:f>IF(AND(U69=TRUE,V69=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA69" s="27" t="str">
+        <x:f>IF(Z69="No","Not comparable",IF(X69&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="20" t="str">
+        <x:v>s10-20261002-05</x:v>
+      </x:c>
+      <x:c r="B70" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C70" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D70" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E70" s="20" t="str">
+        <x:v>Medium Pirate Encounter</x:v>
+      </x:c>
+      <x:c r="F70" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G70" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H70" s="23" t="n">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="I70" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J70" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K70" s="23" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="L70" s="23" t="n">
+        <x:v>2985</x:v>
+      </x:c>
+      <x:c r="M70" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N70" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O70" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P70" s="23" t="n">
+        <x:v>9907346</x:v>
+      </x:c>
+      <x:c r="Q70" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R70" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S70" s="23" t="n">
+        <x:v>6842000</x:v>
+      </x:c>
+      <x:c r="T70" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U70" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V70" s="25" t="n">
+        <x:f>N70+1.5*O70+3*P70+3*Q70</x:f>
+        <x:v>29722038</x:v>
+      </x:c>
+      <x:c r="W70" s="25" t="n">
+        <x:f>S70*3</x:f>
+        <x:v>20526000</x:v>
+      </x:c>
+      <x:c r="X70" s="25" t="n">
+        <x:f>IF(Z70="No",0,V70-W70)</x:f>
+        <x:v>9196038</x:v>
+      </x:c>
+      <x:c r="Y70" s="26" t="n">
+        <x:f>IF(Z70="No",0,IFERROR(V70/W70,0))</x:f>
+        <x:v>1.4480190002923121</x:v>
+      </x:c>
+      <x:c r="Z70" s="27" t="str">
+        <x:f>IF(AND(U70=TRUE,V70=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA70" s="27" t="str">
+        <x:f>IF(Z70="No","Not comparable",IF(X70&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="20" t="str">
+        <x:v>s10-20261002-06</x:v>
+      </x:c>
+      <x:c r="B71" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C71" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D71" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E71" s="20" t="str">
+        <x:v>Small Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F71" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G71" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H71" s="23" t="n">
+        <x:v>668</x:v>
+      </x:c>
+      <x:c r="I71" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J71" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K71" s="23" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="L71" s="23" t="n">
+        <x:v>3080</x:v>
+      </x:c>
+      <x:c r="M71" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N71" s="23" t="n">
+        <x:v>161310632</x:v>
+      </x:c>
+      <x:c r="O71" s="23" t="n">
+        <x:v>54411605</x:v>
+      </x:c>
+      <x:c r="P71" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q71" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R71" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S71" s="23" t="n">
+        <x:v>25307000</x:v>
+      </x:c>
+      <x:c r="T71" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U71" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V71" s="25" t="n">
+        <x:f>N71+1.5*O71+3*P71+3*Q71</x:f>
+        <x:v>242928039.5</x:v>
+      </x:c>
+      <x:c r="W71" s="25" t="n">
+        <x:f>S71*3</x:f>
+        <x:v>75921000</x:v>
+      </x:c>
+      <x:c r="X71" s="25" t="n">
+        <x:f>IF(Z71="No",0,V71-W71)</x:f>
+        <x:v>167007039.5</x:v>
+      </x:c>
+      <x:c r="Y71" s="26" t="n">
+        <x:f>IF(Z71="No",0,IFERROR(V71/W71,0))</x:f>
+        <x:v>3.1997476258215776</x:v>
+      </x:c>
+      <x:c r="Z71" s="27" t="str">
+        <x:f>IF(AND(U71=TRUE,V71=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA71" s="27" t="str">
+        <x:f>IF(Z71="No","Not comparable",IF(X71&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="20" t="str">
+        <x:v>s10-20261002-07</x:v>
+      </x:c>
+      <x:c r="B72" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C72" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D72" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E72" s="20" t="str">
+        <x:v>Small Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F72" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G72" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H72" s="23" t="n">
+        <x:v>599</x:v>
+      </x:c>
+      <x:c r="I72" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J72" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K72" s="23" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="L72" s="23" t="n">
+        <x:v>3555</x:v>
+      </x:c>
+      <x:c r="M72" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N72" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O72" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P72" s="23" t="n">
+        <x:v>8449691</x:v>
+      </x:c>
+      <x:c r="Q72" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R72" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S72" s="23" t="n">
+        <x:v>6808000</x:v>
+      </x:c>
+      <x:c r="T72" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U72" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V72" s="25" t="n">
+        <x:f>N72+1.5*O72+3*P72+3*Q72</x:f>
+        <x:v>25349073</x:v>
+      </x:c>
+      <x:c r="W72" s="25" t="n">
+        <x:f>S72*3</x:f>
+        <x:v>20424000</x:v>
+      </x:c>
+      <x:c r="X72" s="25" t="n">
+        <x:f>IF(Z72="No",0,V72-W72)</x:f>
+        <x:v>4925073</x:v>
+      </x:c>
+      <x:c r="Y72" s="26" t="n">
+        <x:f>IF(Z72="No",0,IFERROR(V72/W72,0))</x:f>
+        <x:v>1.2411414512338426</x:v>
+      </x:c>
+      <x:c r="Z72" s="27" t="str">
+        <x:f>IF(AND(U72=TRUE,V72=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA72" s="27" t="str">
+        <x:f>IF(Z72="No","Not comparable",IF(X72&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="20" t="str">
+        <x:v>s10-20261002-08</x:v>
+      </x:c>
+      <x:c r="B73" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C73" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D73" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E73" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F73" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G73" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H73" s="23" t="n">
+        <x:v>732</x:v>
+      </x:c>
+      <x:c r="I73" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J73" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K73" s="23" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L73" s="23" t="n">
+        <x:v>3080</x:v>
+      </x:c>
+      <x:c r="M73" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N73" s="23" t="n">
+        <x:v>66588378</x:v>
+      </x:c>
+      <x:c r="O73" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P73" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q73" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R73" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S73" s="23" t="n">
+        <x:v>4159000</x:v>
+      </x:c>
+      <x:c r="T73" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U73" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V73" s="25" t="n">
+        <x:f>N73+1.5*O73+3*P73+3*Q73</x:f>
+        <x:v>66588378</x:v>
+      </x:c>
+      <x:c r="W73" s="25" t="n">
+        <x:f>S73*3</x:f>
+        <x:v>12477000</x:v>
+      </x:c>
+      <x:c r="X73" s="25" t="n">
+        <x:f>IF(Z73="No",0,V73-W73)</x:f>
+        <x:v>54111378</x:v>
+      </x:c>
+      <x:c r="Y73" s="26" t="n">
+        <x:f>IF(Z73="No",0,IFERROR(V73/W73,0))</x:f>
+        <x:v>5.3368901178167825</x:v>
+      </x:c>
+      <x:c r="Z73" s="27" t="str">
+        <x:f>IF(AND(U73=TRUE,V73=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA73" s="27" t="str">
+        <x:f>IF(Z73="No","Not comparable",IF(X73&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="20" t="str">
+        <x:v>s10-20261002-09</x:v>
+      </x:c>
+      <x:c r="B74" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C74" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D74" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E74" s="20" t="str">
+        <x:v>Lost Debris Field</x:v>
+      </x:c>
+      <x:c r="F74" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G74" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H74" s="23" t="n">
+        <x:v>682</x:v>
+      </x:c>
+      <x:c r="I74" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J74" s="23" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K74" s="23" t="n">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="L74" s="23" t="n">
+        <x:v>3555</x:v>
+      </x:c>
+      <x:c r="M74" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N74" s="23" t="n">
+        <x:v>34061184</x:v>
+      </x:c>
+      <x:c r="O74" s="23" t="n">
+        <x:v>15165690</x:v>
+      </x:c>
+      <x:c r="P74" s="23" t="n">
+        <x:v>5088183</x:v>
+      </x:c>
+      <x:c r="Q74" s="23" t="n">
+        <x:v>7569152</x:v>
+      </x:c>
+      <x:c r="R74" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S74" s="23" t="n">
+        <x:v>7751000</x:v>
+      </x:c>
+      <x:c r="T74" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U74" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V74" s="25" t="n">
+        <x:f>N74+1.5*O74+3*P74+3*Q74</x:f>
+        <x:v>94781724</x:v>
+      </x:c>
+      <x:c r="W74" s="25" t="n">
+        <x:f>S74*3</x:f>
+        <x:v>23253000</x:v>
+      </x:c>
+      <x:c r="X74" s="25" t="n">
+        <x:f>IF(Z74="No",0,V74-W74)</x:f>
+        <x:v>71528724</x:v>
+      </x:c>
+      <x:c r="Y74" s="26" t="n">
+        <x:f>IF(Z74="No",0,IFERROR(V74/W74,0))</x:f>
+        <x:v>4.076107340988259</x:v>
+      </x:c>
+      <x:c r="Z74" s="27" t="str">
+        <x:f>IF(AND(U74=TRUE,V74=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA74" s="27" t="str">
+        <x:f>IF(Z74="No","Not comparable",IF(X74&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="20" t="str">
+        <x:v>s10-20261002-10</x:v>
+      </x:c>
+      <x:c r="B75" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C75" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D75" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E75" s="20" t="str">
+        <x:v>Small Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F75" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G75" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H75" s="23" t="n">
+        <x:v>681</x:v>
+      </x:c>
+      <x:c r="I75" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J75" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K75" s="23" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="L75" s="23" t="n">
+        <x:v>2890</x:v>
+      </x:c>
+      <x:c r="M75" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N75" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O75" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P75" s="23" t="n">
+        <x:v>34812976</x:v>
+      </x:c>
+      <x:c r="Q75" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R75" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S75" s="23" t="n">
+        <x:v>7740000</x:v>
+      </x:c>
+      <x:c r="T75" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U75" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V75" s="25" t="n">
+        <x:f>N75+1.5*O75+3*P75+3*Q75</x:f>
+        <x:v>104438928</x:v>
+      </x:c>
+      <x:c r="W75" s="25" t="n">
+        <x:f>S75*3</x:f>
+        <x:v>23220000</x:v>
+      </x:c>
+      <x:c r="X75" s="25" t="n">
+        <x:f>IF(Z75="No",0,V75-W75)</x:f>
+        <x:v>81218928</x:v>
+      </x:c>
+      <x:c r="Y75" s="26" t="n">
+        <x:f>IF(Z75="No",0,IFERROR(V75/W75,0))</x:f>
+        <x:v>4.4978005167958655</x:v>
+      </x:c>
+      <x:c r="Z75" s="27" t="str">
+        <x:f>IF(AND(U75=TRUE,V75=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA75" s="27" t="str">
+        <x:f>IF(Z75="No","Not comparable",IF(X75&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="20" t="str">
+        <x:v>s10-20261002-11</x:v>
+      </x:c>
+      <x:c r="B76" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C76" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D76" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E76" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F76" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G76" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H76" s="23" t="n">
+        <x:v>538</x:v>
+      </x:c>
+      <x:c r="I76" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J76" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K76" s="23" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L76" s="23" t="n">
+        <x:v>3650</x:v>
+      </x:c>
+      <x:c r="M76" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N76" s="23" t="n">
+        <x:v>345463360</x:v>
+      </x:c>
+      <x:c r="O76" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P76" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q76" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R76" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S76" s="23" t="n">
+        <x:v>20382000</x:v>
+      </x:c>
+      <x:c r="T76" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U76" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V76" s="25" t="n">
+        <x:f>N76+1.5*O76+3*P76+3*Q76</x:f>
+        <x:v>345463360</x:v>
+      </x:c>
+      <x:c r="W76" s="25" t="n">
+        <x:f>S76*3</x:f>
+        <x:v>61146000</x:v>
+      </x:c>
+      <x:c r="X76" s="25" t="n">
+        <x:f>IF(Z76="No",0,V76-W76)</x:f>
+        <x:v>284317360</x:v>
+      </x:c>
+      <x:c r="Y76" s="26" t="n">
+        <x:f>IF(Z76="No",0,IFERROR(V76/W76,0))</x:f>
+        <x:v>5.649811271383246</x:v>
+      </x:c>
+      <x:c r="Z76" s="27" t="str">
+        <x:f>IF(AND(U76=TRUE,V76=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA76" s="27" t="str">
+        <x:f>IF(Z76="No","Not comparable",IF(X76&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="20" t="str">
+        <x:v>s10-20261002-12</x:v>
+      </x:c>
+      <x:c r="B77" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C77" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D77" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E77" s="20" t="str">
+        <x:v>Medium Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F77" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G77" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H77" s="23" t="n">
+        <x:v>663</x:v>
+      </x:c>
+      <x:c r="I77" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J77" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K77" s="23" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="L77" s="23" t="n">
+        <x:v>3365</x:v>
+      </x:c>
+      <x:c r="M77" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N77" s="23" t="n">
+        <x:v>20498057</x:v>
+      </x:c>
+      <x:c r="O77" s="23" t="n">
+        <x:v>13828378</x:v>
+      </x:c>
+      <x:c r="P77" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q77" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R77" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S77" s="23" t="n">
+        <x:v>2511000</x:v>
+      </x:c>
+      <x:c r="T77" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U77" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V77" s="25" t="n">
+        <x:f>N77+1.5*O77+3*P77+3*Q77</x:f>
+        <x:v>41240624</x:v>
+      </x:c>
+      <x:c r="W77" s="25" t="n">
+        <x:f>S77*3</x:f>
+        <x:v>7533000</x:v>
+      </x:c>
+      <x:c r="X77" s="25" t="n">
+        <x:f>IF(Z77="No",0,V77-W77)</x:f>
+        <x:v>33707624</x:v>
+      </x:c>
+      <x:c r="Y77" s="26" t="n">
+        <x:f>IF(Z77="No",0,IFERROR(V77/W77,0))</x:f>
+        <x:v>5.474661356697199</x:v>
+      </x:c>
+      <x:c r="Z77" s="27" t="str">
+        <x:f>IF(AND(U77=TRUE,V77=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA77" s="27" t="str">
+        <x:f>IF(Z77="No","Not comparable",IF(X77&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="20" t="str">
+        <x:v>s50-20261002-01</x:v>
+      </x:c>
+      <x:c r="B78" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C78" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D78" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E78" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F78" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G78" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H78" s="23" t="n">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="I78" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J78" s="23" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K78" s="23" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="L78" s="23" t="n">
+        <x:v>6215</x:v>
+      </x:c>
+      <x:c r="M78" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N78" s="23" t="n">
+        <x:v>166610082</x:v>
+      </x:c>
+      <x:c r="O78" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P78" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q78" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R78" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S78" s="23" t="n">
+        <x:v>25277000</x:v>
+      </x:c>
+      <x:c r="T78" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U78" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V78" s="25" t="n">
+        <x:f>N78+1.5*O78+3*P78+3*Q78</x:f>
+        <x:v>166610082</x:v>
+      </x:c>
+      <x:c r="W78" s="25" t="n">
+        <x:f>S78*3</x:f>
+        <x:v>75831000</x:v>
+      </x:c>
+      <x:c r="X78" s="25" t="n">
+        <x:f>IF(Z78="No",0,V78-W78)</x:f>
+        <x:v>90779082</x:v>
+      </x:c>
+      <x:c r="Y78" s="26" t="n">
+        <x:f>IF(Z78="No",0,IFERROR(V78/W78,0))</x:f>
+        <x:v>2.197123630177632</x:v>
+      </x:c>
+      <x:c r="Z78" s="27" t="str">
+        <x:f>IF(AND(U78=TRUE,V78=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA78" s="27" t="str">
+        <x:f>IF(Z78="No","Not comparable",IF(X78&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="20" t="str">
+        <x:v>s50-20261002-02</x:v>
+      </x:c>
+      <x:c r="B79" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C79" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D79" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E79" s="20" t="str">
+        <x:v>Mysterious Nebula</x:v>
+      </x:c>
+      <x:c r="F79" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G79" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H79" s="23" t="n">
+        <x:v>597</x:v>
+      </x:c>
+      <x:c r="I79" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J79" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K79" s="23" t="n">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="L79" s="23" t="n">
+        <x:v>3175</x:v>
+      </x:c>
+      <x:c r="M79" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N79" s="23" t="n">
+        <x:v>14641794</x:v>
+      </x:c>
+      <x:c r="O79" s="23" t="n">
+        <x:v>6519237</x:v>
+      </x:c>
+      <x:c r="P79" s="23" t="n">
+        <x:v>2187245</x:v>
+      </x:c>
+      <x:c r="Q79" s="23" t="n">
+        <x:v>13014928</x:v>
+      </x:c>
+      <x:c r="R79" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S79" s="23" t="n">
+        <x:v>22617000</x:v>
+      </x:c>
+      <x:c r="T79" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U79" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V79" s="25" t="n">
+        <x:f>N79+1.5*O79+3*P79+3*Q79</x:f>
+        <x:v>70027168.5</x:v>
+      </x:c>
+      <x:c r="W79" s="25" t="n">
+        <x:f>S79*3</x:f>
+        <x:v>67851000</x:v>
+      </x:c>
+      <x:c r="X79" s="25" t="n">
+        <x:f>IF(Z79="No",0,V79-W79)</x:f>
+        <x:v>2176168.5</x:v>
+      </x:c>
+      <x:c r="Y79" s="26" t="n">
+        <x:f>IF(Z79="No",0,IFERROR(V79/W79,0))</x:f>
+        <x:v>1.0320727550072955</x:v>
+      </x:c>
+      <x:c r="Z79" s="27" t="str">
+        <x:f>IF(AND(U79=TRUE,V79=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA79" s="27" t="str">
+        <x:f>IF(Z79="No","Not comparable",IF(X79&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="20" t="str">
+        <x:v>s50-20261002-03</x:v>
+      </x:c>
+      <x:c r="B80" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C80" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D80" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E80" s="20" t="str">
+        <x:v>Rescue</x:v>
+      </x:c>
+      <x:c r="F80" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G80" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H80" s="23" t="n">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="I80" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J80" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K80" s="23" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L80" s="23" t="n">
+        <x:v>3840</x:v>
+      </x:c>
+      <x:c r="M80" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N80" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O80" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P80" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q80" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R80" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S80" s="23" t="n">
+        <x:v>2185000</x:v>
+      </x:c>
+      <x:c r="T80" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U80" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V80" s="25" t="n">
+        <x:f>N80+1.5*O80+3*P80+3*Q80</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W80" s="25" t="n">
+        <x:f>S80*3</x:f>
+        <x:v>6555000</x:v>
+      </x:c>
+      <x:c r="X80" s="25" t="n">
+        <x:f>IF(Z80="No",0,V80-W80)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y80" s="26" t="n">
+        <x:f>IF(Z80="No",0,IFERROR(V80/W80,0))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z80" s="27" t="str">
+        <x:f>IF(AND(U80=TRUE,V80=0),"No","Yes")</x:f>
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AA80" s="27" t="str">
+        <x:f>IF(Z80="No","Not comparable",IF(X80&gt;0,"Yes","No"))</x:f>
+        <x:v>Not comparable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="20" t="str">
+        <x:v>s50-20261002-04</x:v>
+      </x:c>
+      <x:c r="B81" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C81" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D81" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E81" s="20" t="str">
+        <x:v>Delivery: Deuterium</x:v>
+      </x:c>
+      <x:c r="F81" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G81" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H81" s="23" t="n">
+        <x:v>566</x:v>
+      </x:c>
+      <x:c r="I81" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J81" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K81" s="23" t="n">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="L81" s="23" t="n">
+        <x:v>4505</x:v>
+      </x:c>
+      <x:c r="M81" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N81" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O81" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P81" s="23" t="n">
+        <x:v>81320370</x:v>
+      </x:c>
+      <x:c r="Q81" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R81" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S81" s="23" t="n">
+        <x:v>10721000</x:v>
+      </x:c>
+      <x:c r="T81" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U81" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V81" s="25" t="n">
+        <x:f>N81+1.5*O81+3*P81+3*Q81</x:f>
+        <x:v>243961110</x:v>
+      </x:c>
+      <x:c r="W81" s="25" t="n">
+        <x:f>S81*3</x:f>
+        <x:v>32163000</x:v>
+      </x:c>
+      <x:c r="X81" s="25" t="n">
+        <x:f>IF(Z81="No",0,V81-W81)</x:f>
+        <x:v>211798110</x:v>
+      </x:c>
+      <x:c r="Y81" s="26" t="n">
+        <x:f>IF(Z81="No",0,IFERROR(V81/W81,0))</x:f>
+        <x:v>7.585147840686503</x:v>
+      </x:c>
+      <x:c r="Z81" s="27" t="str">
+        <x:f>IF(AND(U81=TRUE,V81=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA81" s="27" t="str">
+        <x:f>IF(Z81="No","Not comparable",IF(X81&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="20" t="str">
+        <x:v>s50-20261002-05</x:v>
+      </x:c>
+      <x:c r="B82" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C82" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D82" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E82" s="20" t="str">
+        <x:v>Pirate Hideout</x:v>
+      </x:c>
+      <x:c r="F82" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G82" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H82" s="23" t="n">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="I82" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J82" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K82" s="23" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="L82" s="23" t="n">
+        <x:v>4695</x:v>
+      </x:c>
+      <x:c r="M82" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N82" s="23" t="n">
+        <x:v>17423820</x:v>
+      </x:c>
+      <x:c r="O82" s="23" t="n">
+        <x:v>7757930</x:v>
+      </x:c>
+      <x:c r="P82" s="23" t="n">
+        <x:v>2602834</x:v>
+      </x:c>
+      <x:c r="Q82" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R82" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S82" s="23" t="n">
+        <x:v>3773000</x:v>
+      </x:c>
+      <x:c r="T82" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U82" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V82" s="25" t="n">
+        <x:f>N82+1.5*O82+3*P82+3*Q82</x:f>
+        <x:v>36869217</x:v>
+      </x:c>
+      <x:c r="W82" s="25" t="n">
+        <x:f>S82*3</x:f>
+        <x:v>11319000</x:v>
+      </x:c>
+      <x:c r="X82" s="25" t="n">
+        <x:f>IF(Z82="No",0,V82-W82)</x:f>
+        <x:v>25550217</x:v>
+      </x:c>
+      <x:c r="Y82" s="26" t="n">
+        <x:f>IF(Z82="No",0,IFERROR(V82/W82,0))</x:f>
+        <x:v>3.257285714285714</x:v>
+      </x:c>
+      <x:c r="Z82" s="27" t="str">
+        <x:f>IF(AND(U82=TRUE,V82=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA82" s="27" t="str">
+        <x:f>IF(Z82="No","Not comparable",IF(X82&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="20" t="str">
+        <x:v>s50-20261002-06</x:v>
+      </x:c>
+      <x:c r="B83" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C83" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D83" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E83" s="20" t="str">
+        <x:v>Mysterious Nebula</x:v>
+      </x:c>
+      <x:c r="F83" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G83" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H83" s="23" t="n">
+        <x:v>683</x:v>
+      </x:c>
+      <x:c r="I83" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J83" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K83" s="23" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="L83" s="23" t="n">
+        <x:v>6120</x:v>
+      </x:c>
+      <x:c r="M83" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N83" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O83" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P83" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q83" s="23" t="n">
+        <x:v>5380623</x:v>
+      </x:c>
+      <x:c r="R83" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S83" s="23" t="n">
+        <x:v>11644000</x:v>
+      </x:c>
+      <x:c r="T83" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U83" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V83" s="25" t="n">
+        <x:f>N83+1.5*O83+3*P83+3*Q83</x:f>
+        <x:v>16141869</x:v>
+      </x:c>
+      <x:c r="W83" s="25" t="n">
+        <x:f>S83*3</x:f>
+        <x:v>34932000</x:v>
+      </x:c>
+      <x:c r="X83" s="25" t="n">
+        <x:f>IF(Z83="No",0,V83-W83)</x:f>
+        <x:v>-18790131</x:v>
+      </x:c>
+      <x:c r="Y83" s="26" t="n">
+        <x:f>IF(Z83="No",0,IFERROR(V83/W83,0))</x:f>
+        <x:v>0.46209403984884917</x:v>
+      </x:c>
+      <x:c r="Z83" s="27" t="str">
+        <x:f>IF(AND(U83=TRUE,V83=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA83" s="27" t="str">
+        <x:f>IF(Z83="No","Not comparable",IF(X83&gt;0,"Yes","No"))</x:f>
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="20" t="str">
+        <x:v>s50-20261002-07</x:v>
+      </x:c>
+      <x:c r="B84" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C84" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D84" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E84" s="20" t="str">
+        <x:v>Chaos Mission</x:v>
+      </x:c>
+      <x:c r="F84" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G84" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H84" s="23" t="n">
+        <x:v>598</x:v>
+      </x:c>
+      <x:c r="I84" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J84" s="23" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K84" s="23" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="L84" s="23" t="n">
+        <x:v>3840</x:v>
+      </x:c>
+      <x:c r="M84" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N84" s="23" t="n">
+        <x:v>45383520</x:v>
+      </x:c>
+      <x:c r="O84" s="23" t="n">
+        <x:v>20206944</x:v>
+      </x:c>
+      <x:c r="P84" s="23" t="n">
+        <x:v>6779556</x:v>
+      </x:c>
+      <x:c r="Q84" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R84" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S84" s="23" t="n">
+        <x:v>10194000</x:v>
+      </x:c>
+      <x:c r="T84" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U84" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V84" s="25" t="n">
+        <x:f>N84+1.5*O84+3*P84+3*Q84</x:f>
+        <x:v>96032604</x:v>
+      </x:c>
+      <x:c r="W84" s="25" t="n">
+        <x:f>S84*3</x:f>
+        <x:v>30582000</x:v>
+      </x:c>
+      <x:c r="X84" s="25" t="n">
+        <x:f>IF(Z84="No",0,V84-W84)</x:f>
+        <x:v>65450604</x:v>
+      </x:c>
+      <x:c r="Y84" s="26" t="n">
+        <x:f>IF(Z84="No",0,IFERROR(V84/W84,0))</x:f>
+        <x:v>3.1401675495389445</x:v>
+      </x:c>
+      <x:c r="Z84" s="27" t="str">
+        <x:f>IF(AND(U84=TRUE,V84=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA84" s="27" t="str">
+        <x:f>IF(Z84="No","Not comparable",IF(X84&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="20" t="str">
+        <x:v>s50-20261002-08</x:v>
+      </x:c>
+      <x:c r="B85" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C85" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D85" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E85" s="20" t="str">
+        <x:v>Medium Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F85" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G85" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H85" s="23" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="I85" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J85" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K85" s="23" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="L85" s="23" t="n">
+        <x:v>2985</x:v>
+      </x:c>
+      <x:c r="M85" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N85" s="23" t="n">
+        <x:v>75628082</x:v>
+      </x:c>
+      <x:c r="O85" s="23" t="n">
+        <x:v>84693428</x:v>
+      </x:c>
+      <x:c r="P85" s="23" t="n">
+        <x:v>11297602</x:v>
+      </x:c>
+      <x:c r="Q85" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R85" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S85" s="23" t="n">
+        <x:v>13638000</x:v>
+      </x:c>
+      <x:c r="T85" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U85" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V85" s="25" t="n">
+        <x:f>N85+1.5*O85+3*P85+3*Q85</x:f>
+        <x:v>236561030</x:v>
+      </x:c>
+      <x:c r="W85" s="25" t="n">
+        <x:f>S85*3</x:f>
+        <x:v>40914000</x:v>
+      </x:c>
+      <x:c r="X85" s="25" t="n">
+        <x:f>IF(Z85="No",0,V85-W85)</x:f>
+        <x:v>195647030</x:v>
+      </x:c>
+      <x:c r="Y85" s="26" t="n">
+        <x:f>IF(Z85="No",0,IFERROR(V85/W85,0))</x:f>
+        <x:v>5.781909126460381</x:v>
+      </x:c>
+      <x:c r="Z85" s="27" t="str">
+        <x:f>IF(AND(U85=TRUE,V85=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA85" s="27" t="str">
+        <x:f>IF(Z85="No","Not comparable",IF(X85&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="20" t="str">
+        <x:v>s50-20261002-09</x:v>
+      </x:c>
+      <x:c r="B86" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C86" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D86" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E86" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F86" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G86" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H86" s="23" t="n">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="I86" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J86" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K86" s="23" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="L86" s="23" t="n">
+        <x:v>6215</x:v>
+      </x:c>
+      <x:c r="M86" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N86" s="23" t="n">
+        <x:v>63955660</x:v>
+      </x:c>
+      <x:c r="O86" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P86" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q86" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R86" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S86" s="23" t="n">
+        <x:v>10062000</x:v>
+      </x:c>
+      <x:c r="T86" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U86" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V86" s="25" t="n">
+        <x:f>N86+1.5*O86+3*P86+3*Q86</x:f>
+        <x:v>63955660</x:v>
+      </x:c>
+      <x:c r="W86" s="25" t="n">
+        <x:f>S86*3</x:f>
+        <x:v>30186000</x:v>
+      </x:c>
+      <x:c r="X86" s="25" t="n">
+        <x:f>IF(Z86="No",0,V86-W86)</x:f>
+        <x:v>33769660</x:v>
+      </x:c>
+      <x:c r="Y86" s="26" t="n">
+        <x:f>IF(Z86="No",0,IFERROR(V86/W86,0))</x:f>
+        <x:v>2.118719273835553</x:v>
+      </x:c>
+      <x:c r="Z86" s="27" t="str">
+        <x:f>IF(AND(U86=TRUE,V86=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA86" s="27" t="str">
+        <x:f>IF(Z86="No","Not comparable",IF(X86&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="20" t="str">
+        <x:v>s50-20261002-10</x:v>
+      </x:c>
+      <x:c r="B87" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C87" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D87" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E87" s="20" t="str">
+        <x:v>Delivery: Crystal</x:v>
+      </x:c>
+      <x:c r="F87" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G87" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H87" s="23" t="n">
+        <x:v>620</x:v>
+      </x:c>
+      <x:c r="I87" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J87" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K87" s="23" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="L87" s="23" t="n">
+        <x:v>6215</x:v>
+      </x:c>
+      <x:c r="M87" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N87" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O87" s="23" t="n">
+        <x:v>76936330</x:v>
+      </x:c>
+      <x:c r="P87" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q87" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R87" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S87" s="23" t="n">
+        <x:v>17616000</x:v>
+      </x:c>
+      <x:c r="T87" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U87" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V87" s="25" t="n">
+        <x:f>N87+1.5*O87+3*P87+3*Q87</x:f>
+        <x:v>115404495</x:v>
+      </x:c>
+      <x:c r="W87" s="25" t="n">
+        <x:f>S87*3</x:f>
+        <x:v>52848000</x:v>
+      </x:c>
+      <x:c r="X87" s="25" t="n">
+        <x:f>IF(Z87="No",0,V87-W87)</x:f>
+        <x:v>62556495</x:v>
+      </x:c>
+      <x:c r="Y87" s="26" t="n">
+        <x:f>IF(Z87="No",0,IFERROR(V87/W87,0))</x:f>
+        <x:v>2.183706005903724</x:v>
+      </x:c>
+      <x:c r="Z87" s="27" t="str">
+        <x:f>IF(AND(U87=TRUE,V87=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA87" s="27" t="str">
+        <x:f>IF(Z87="No","Not comparable",IF(X87&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="20" t="str">
+        <x:v>s50-20261002-11</x:v>
+      </x:c>
+      <x:c r="B88" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C88" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D88" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E88" s="20" t="str">
+        <x:v>Chaos Mission</x:v>
+      </x:c>
+      <x:c r="F88" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G88" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H88" s="23" t="n">
+        <x:v>704</x:v>
+      </x:c>
+      <x:c r="I88" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J88" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K88" s="23" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="L88" s="23" t="n">
+        <x:v>2985</x:v>
+      </x:c>
+      <x:c r="M88" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N88" s="23" t="n">
+        <x:v>260801628</x:v>
+      </x:c>
+      <x:c r="O88" s="23" t="n">
+        <x:v>116121537</x:v>
+      </x:c>
+      <x:c r="P88" s="23" t="n">
+        <x:v>38959509</x:v>
+      </x:c>
+      <x:c r="Q88" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R88" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S88" s="23" t="n">
+        <x:v>21337000</x:v>
+      </x:c>
+      <x:c r="T88" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U88" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V88" s="25" t="n">
+        <x:f>N88+1.5*O88+3*P88+3*Q88</x:f>
+        <x:v>551862460.5</x:v>
+      </x:c>
+      <x:c r="W88" s="25" t="n">
+        <x:f>S88*3</x:f>
+        <x:v>64011000</x:v>
+      </x:c>
+      <x:c r="X88" s="25" t="n">
+        <x:f>IF(Z88="No",0,V88-W88)</x:f>
+        <x:v>487851460.5</x:v>
+      </x:c>
+      <x:c r="Y88" s="26" t="n">
+        <x:f>IF(Z88="No",0,IFERROR(V88/W88,0))</x:f>
+        <x:v>8.621369147490276</x:v>
+      </x:c>
+      <x:c r="Z88" s="27" t="str">
+        <x:f>IF(AND(U88=TRUE,V88=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA88" s="27" t="str">
+        <x:f>IF(Z88="No","Not comparable",IF(X88&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="20" t="str">
+        <x:v>s50-20261002-12</x:v>
+      </x:c>
+      <x:c r="B89" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C89" s="22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D89" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E89" s="20" t="str">
+        <x:v>Small Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F89" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G89" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H89" s="23" t="n">
+        <x:v>707</x:v>
+      </x:c>
+      <x:c r="I89" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J89" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K89" s="23" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="L89" s="23" t="n">
+        <x:v>3745</x:v>
+      </x:c>
+      <x:c r="M89" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N89" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O89" s="23" t="n">
+        <x:v>25522102</x:v>
+      </x:c>
+      <x:c r="P89" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q89" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R89" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S89" s="23" t="n">
+        <x:v>13392000</x:v>
+      </x:c>
+      <x:c r="T89" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U89" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V89" s="25" t="n">
+        <x:f>N89+1.5*O89+3*P89+3*Q89</x:f>
+        <x:v>38283153</x:v>
+      </x:c>
+      <x:c r="W89" s="25" t="n">
+        <x:f>S89*3</x:f>
+        <x:v>40176000</x:v>
+      </x:c>
+      <x:c r="X89" s="25" t="n">
+        <x:f>IF(Z89="No",0,V89-W89)</x:f>
+        <x:v>-1892847</x:v>
+      </x:c>
+      <x:c r="Y89" s="26" t="n">
+        <x:f>IF(Z89="No",0,IFERROR(V89/W89,0))</x:f>
+        <x:v>0.9528861260454002</x:v>
+      </x:c>
+      <x:c r="Z89" s="27" t="str">
+        <x:f>IF(AND(U89=TRUE,V89=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA89" s="27" t="str">
+        <x:f>IF(Z89="No","Not comparable",IF(X89&gt;0,"Yes","No"))</x:f>
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="20" t="str">
+        <x:v>s150-20261002-01</x:v>
+      </x:c>
+      <x:c r="B90" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C90" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D90" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E90" s="20" t="str">
+        <x:v>Medium Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F90" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G90" s="23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H90" s="23" t="n">
+        <x:v>531</x:v>
+      </x:c>
+      <x:c r="I90" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J90" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K90" s="23" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="L90" s="23" t="n">
+        <x:v>10490</x:v>
+      </x:c>
+      <x:c r="M90" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N90" s="23" t="n">
+        <x:v>80506442</x:v>
+      </x:c>
+      <x:c r="O90" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P90" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q90" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R90" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S90" s="23" t="n">
+        <x:v>5029000</x:v>
+      </x:c>
+      <x:c r="T90" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U90" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V90" s="25" t="n">
+        <x:f>N90+1.5*O90+3*P90+3*Q90</x:f>
+        <x:v>80506442</x:v>
+      </x:c>
+      <x:c r="W90" s="25" t="n">
+        <x:f>S90*3</x:f>
+        <x:v>15087000</x:v>
+      </x:c>
+      <x:c r="X90" s="25" t="n">
+        <x:f>IF(Z90="No",0,V90-W90)</x:f>
+        <x:v>65419442</x:v>
+      </x:c>
+      <x:c r="Y90" s="26" t="n">
+        <x:f>IF(Z90="No",0,IFERROR(V90/W90,0))</x:f>
+        <x:v>5.336146483727712</x:v>
+      </x:c>
+      <x:c r="Z90" s="27" t="str">
+        <x:f>IF(AND(U90=TRUE,V90=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA90" s="27" t="str">
+        <x:f>IF(Z90="No","Not comparable",IF(X90&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="20" t="str">
+        <x:v>s150-20261002-02</x:v>
+      </x:c>
+      <x:c r="B91" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C91" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D91" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E91" s="20" t="str">
+        <x:v>Medium Pirate Encounter</x:v>
+      </x:c>
+      <x:c r="F91" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G91" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H91" s="23" t="n">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="I91" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J91" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K91" s="23" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="L91" s="23" t="n">
+        <x:v>12200</x:v>
+      </x:c>
+      <x:c r="M91" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N91" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O91" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P91" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q91" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R91" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S91" s="23" t="n">
+        <x:v>9325000</x:v>
+      </x:c>
+      <x:c r="T91" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U91" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V91" s="25" t="n">
+        <x:f>N91+1.5*O91+3*P91+3*Q91</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W91" s="25" t="n">
+        <x:f>S91*3</x:f>
+        <x:v>27975000</x:v>
+      </x:c>
+      <x:c r="X91" s="25" t="n">
+        <x:f>IF(Z91="No",0,V91-W91)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y91" s="26" t="n">
+        <x:f>IF(Z91="No",0,IFERROR(V91/W91,0))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z91" s="27" t="str">
+        <x:f>IF(AND(U91=TRUE,V91=0),"No","Yes")</x:f>
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AA91" s="27" t="str">
+        <x:f>IF(Z91="No","Not comparable",IF(X91&gt;0,"Yes","No"))</x:f>
+        <x:v>Not comparable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="20" t="str">
+        <x:v>s150-20261002-03</x:v>
+      </x:c>
+      <x:c r="B92" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C92" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D92" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E92" s="20" t="str">
+        <x:v>Medium Pirate Encounter</x:v>
+      </x:c>
+      <x:c r="F92" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G92" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H92" s="23" t="n">
+        <x:v>694</x:v>
+      </x:c>
+      <x:c r="I92" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J92" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K92" s="23" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="L92" s="23" t="n">
+        <x:v>7545</x:v>
+      </x:c>
+      <x:c r="M92" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N92" s="23" t="n">
+        <x:v>8665123</x:v>
+      </x:c>
+      <x:c r="O92" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P92" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q92" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R92" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S92" s="23" t="n">
+        <x:v>2629000</x:v>
+      </x:c>
+      <x:c r="T92" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U92" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V92" s="25" t="n">
+        <x:f>N92+1.5*O92+3*P92+3*Q92</x:f>
+        <x:v>8665123</x:v>
+      </x:c>
+      <x:c r="W92" s="25" t="n">
+        <x:f>S92*3</x:f>
+        <x:v>7887000</x:v>
+      </x:c>
+      <x:c r="X92" s="25" t="n">
+        <x:f>IF(Z92="No",0,V92-W92)</x:f>
+        <x:v>778123</x:v>
+      </x:c>
+      <x:c r="Y92" s="26" t="n">
+        <x:f>IF(Z92="No",0,IFERROR(V92/W92,0))</x:f>
+        <x:v>1.0986589324204388</x:v>
+      </x:c>
+      <x:c r="Z92" s="27" t="str">
+        <x:f>IF(AND(U92=TRUE,V92=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA92" s="27" t="str">
+        <x:f>IF(Z92="No","Not comparable",IF(X92&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="20" t="str">
+        <x:v>s150-20261002-04</x:v>
+      </x:c>
+      <x:c r="B93" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C93" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D93" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E93" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F93" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G93" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H93" s="23" t="n">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="I93" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J93" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K93" s="23" t="n">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="L93" s="23" t="n">
+        <x:v>8210</x:v>
+      </x:c>
+      <x:c r="M93" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N93" s="23" t="n">
+        <x:v>75706564</x:v>
+      </x:c>
+      <x:c r="O93" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P93" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q93" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R93" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S93" s="23" t="n">
+        <x:v>11911000</x:v>
+      </x:c>
+      <x:c r="T93" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U93" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V93" s="25" t="n">
+        <x:f>N93+1.5*O93+3*P93+3*Q93</x:f>
+        <x:v>75706564</x:v>
+      </x:c>
+      <x:c r="W93" s="25" t="n">
+        <x:f>S93*3</x:f>
+        <x:v>35733000</x:v>
+      </x:c>
+      <x:c r="X93" s="25" t="n">
+        <x:f>IF(Z93="No",0,V93-W93)</x:f>
+        <x:v>39973564</x:v>
+      </x:c>
+      <x:c r="Y93" s="26" t="n">
+        <x:f>IF(Z93="No",0,IFERROR(V93/W93,0))</x:f>
+        <x:v>2.1186736070299164</x:v>
+      </x:c>
+      <x:c r="Z93" s="27" t="str">
+        <x:f>IF(AND(U93=TRUE,V93=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA93" s="27" t="str">
+        <x:f>IF(Z93="No","Not comparable",IF(X93&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="20" t="str">
+        <x:v>s150-20261002-05</x:v>
+      </x:c>
+      <x:c r="B94" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C94" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D94" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E94" s="20" t="str">
+        <x:v>Resource: Deuterium</x:v>
+      </x:c>
+      <x:c r="F94" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G94" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H94" s="23" t="n">
+        <x:v>724</x:v>
+      </x:c>
+      <x:c r="I94" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J94" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K94" s="23" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="L94" s="23" t="n">
+        <x:v>3935</x:v>
+      </x:c>
+      <x:c r="M94" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N94" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O94" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P94" s="23" t="n">
+        <x:v>81703872</x:v>
+      </x:c>
+      <x:c r="Q94" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R94" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S94" s="23" t="n">
+        <x:v>10971000</x:v>
+      </x:c>
+      <x:c r="T94" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U94" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V94" s="25" t="n">
+        <x:f>N94+1.5*O94+3*P94+3*Q94</x:f>
+        <x:v>245111616</x:v>
+      </x:c>
+      <x:c r="W94" s="25" t="n">
+        <x:f>S94*3</x:f>
+        <x:v>32913000</x:v>
+      </x:c>
+      <x:c r="X94" s="25" t="n">
+        <x:f>IF(Z94="No",0,V94-W94)</x:f>
+        <x:v>212198616</x:v>
+      </x:c>
+      <x:c r="Y94" s="26" t="n">
+        <x:f>IF(Z94="No",0,IFERROR(V94/W94,0))</x:f>
+        <x:v>7.447258408531583</x:v>
+      </x:c>
+      <x:c r="Z94" s="27" t="str">
+        <x:f>IF(AND(U94=TRUE,V94=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA94" s="27" t="str">
+        <x:f>IF(Z94="No","Not comparable",IF(X94&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="20" t="str">
+        <x:v>s150-20261002-06</x:v>
+      </x:c>
+      <x:c r="B95" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C95" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D95" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E95" s="20" t="str">
+        <x:v>Resource: Deuterium</x:v>
+      </x:c>
+      <x:c r="F95" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G95" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H95" s="23" t="n">
+        <x:v>632</x:v>
+      </x:c>
+      <x:c r="I95" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J95" s="23" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K95" s="23" t="n">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="L95" s="23" t="n">
+        <x:v>15620</x:v>
+      </x:c>
+      <x:c r="M95" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N95" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O95" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P95" s="23" t="n">
+        <x:v>98810124</x:v>
+      </x:c>
+      <x:c r="Q95" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R95" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S95" s="23" t="n">
+        <x:v>33521000</x:v>
+      </x:c>
+      <x:c r="T95" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U95" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V95" s="25" t="n">
+        <x:f>N95+1.5*O95+3*P95+3*Q95</x:f>
+        <x:v>296430372</x:v>
+      </x:c>
+      <x:c r="W95" s="25" t="n">
+        <x:f>S95*3</x:f>
+        <x:v>100563000</x:v>
+      </x:c>
+      <x:c r="X95" s="25" t="n">
+        <x:f>IF(Z95="No",0,V95-W95)</x:f>
+        <x:v>195867372</x:v>
+      </x:c>
+      <x:c r="Y95" s="26" t="n">
+        <x:f>IF(Z95="No",0,IFERROR(V95/W95,0))</x:f>
+        <x:v>2.9477081232660125</x:v>
+      </x:c>
+      <x:c r="Z95" s="27" t="str">
+        <x:f>IF(AND(U95=TRUE,V95=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA95" s="27" t="str">
+        <x:f>IF(Z95="No","Not comparable",IF(X95&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="20" t="str">
+        <x:v>s150-20261002-07</x:v>
+      </x:c>
+      <x:c r="B96" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C96" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D96" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E96" s="20" t="str">
+        <x:v>Resource: Crystal</x:v>
+      </x:c>
+      <x:c r="F96" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G96" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H96" s="23" t="n">
+        <x:v>585</x:v>
+      </x:c>
+      <x:c r="I96" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J96" s="23" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K96" s="23" t="n">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="L96" s="23" t="n">
+        <x:v>12200</x:v>
+      </x:c>
+      <x:c r="M96" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N96" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O96" s="23" t="n">
+        <x:v>187246339</x:v>
+      </x:c>
+      <x:c r="P96" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q96" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R96" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S96" s="23" t="n">
+        <x:v>15514000</x:v>
+      </x:c>
+      <x:c r="T96" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U96" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V96" s="25" t="n">
+        <x:f>N96+1.5*O96+3*P96+3*Q96</x:f>
+        <x:v>280869508.5</x:v>
+      </x:c>
+      <x:c r="W96" s="25" t="n">
+        <x:f>S96*3</x:f>
+        <x:v>46542000</x:v>
+      </x:c>
+      <x:c r="X96" s="25" t="n">
+        <x:f>IF(Z96="No",0,V96-W96)</x:f>
+        <x:v>234327508.5</x:v>
+      </x:c>
+      <x:c r="Y96" s="26" t="n">
+        <x:f>IF(Z96="No",0,IFERROR(V96/W96,0))</x:f>
+        <x:v>6.034753738558721</x:v>
+      </x:c>
+      <x:c r="Z96" s="27" t="str">
+        <x:f>IF(AND(U96=TRUE,V96=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA96" s="27" t="str">
+        <x:f>IF(Z96="No","Not comparable",IF(X96&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="20" t="str">
+        <x:v>s150-20261002-08</x:v>
+      </x:c>
+      <x:c r="B97" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C97" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D97" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E97" s="20" t="str">
+        <x:v>Rescue</x:v>
+      </x:c>
+      <x:c r="F97" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G97" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H97" s="23" t="n">
+        <x:v>634</x:v>
+      </x:c>
+      <x:c r="I97" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J97" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K97" s="23" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L97" s="23" t="n">
+        <x:v>11630</x:v>
+      </x:c>
+      <x:c r="M97" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N97" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O97" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P97" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q97" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R97" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S97" s="23" t="n">
+        <x:v>1200000</x:v>
+      </x:c>
+      <x:c r="T97" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U97" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V97" s="25" t="n">
+        <x:f>N97+1.5*O97+3*P97+3*Q97</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W97" s="25" t="n">
+        <x:f>S97*3</x:f>
+        <x:v>3600000</x:v>
+      </x:c>
+      <x:c r="X97" s="25" t="n">
+        <x:f>IF(Z97="No",0,V97-W97)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y97" s="26" t="n">
+        <x:f>IF(Z97="No",0,IFERROR(V97/W97,0))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z97" s="27" t="str">
+        <x:f>IF(AND(U97=TRUE,V97=0),"No","Yes")</x:f>
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AA97" s="27" t="str">
+        <x:f>IF(Z97="No","Not comparable",IF(X97&gt;0,"Yes","No"))</x:f>
+        <x:v>Not comparable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="20" t="str">
+        <x:v>s150-20261002-09</x:v>
+      </x:c>
+      <x:c r="B98" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C98" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D98" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E98" s="20" t="str">
+        <x:v>Small Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F98" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G98" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H98" s="23" t="n">
+        <x:v>713</x:v>
+      </x:c>
+      <x:c r="I98" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J98" s="23" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K98" s="23" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="L98" s="23" t="n">
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="M98" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N98" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O98" s="23" t="n">
+        <x:v>3891882</x:v>
+      </x:c>
+      <x:c r="P98" s="23" t="n">
+        <x:v>2534693</x:v>
+      </x:c>
+      <x:c r="Q98" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R98" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S98" s="23" t="n">
+        <x:v>3005000</x:v>
+      </x:c>
+      <x:c r="T98" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U98" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V98" s="25" t="n">
+        <x:f>N98+1.5*O98+3*P98+3*Q98</x:f>
+        <x:v>13441902</x:v>
+      </x:c>
+      <x:c r="W98" s="25" t="n">
+        <x:f>S98*3</x:f>
+        <x:v>9015000</x:v>
+      </x:c>
+      <x:c r="X98" s="25" t="n">
+        <x:f>IF(Z98="No",0,V98-W98)</x:f>
+        <x:v>4426902</x:v>
+      </x:c>
+      <x:c r="Y98" s="26" t="n">
+        <x:f>IF(Z98="No",0,IFERROR(V98/W98,0))</x:f>
+        <x:v>1.4910595673876872</x:v>
+      </x:c>
+      <x:c r="Z98" s="27" t="str">
+        <x:f>IF(AND(U98=TRUE,V98=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA98" s="27" t="str">
+        <x:f>IF(Z98="No","Not comparable",IF(X98&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="20" t="str">
+        <x:v>s150-20261002-10</x:v>
+      </x:c>
+      <x:c r="B99" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C99" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D99" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E99" s="20" t="str">
+        <x:v>Alien Encounter</x:v>
+      </x:c>
+      <x:c r="F99" s="20" t="str">
+        <x:v>PvP</x:v>
+      </x:c>
+      <x:c r="G99" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H99" s="23" t="n">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="I99" s="23" t="str">
+        <x:v>Combat</x:v>
+      </x:c>
+      <x:c r="J99" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K99" s="23" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="L99" s="23" t="n">
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="M99" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N99" s="23" t="n">
+        <x:v>34162460</x:v>
+      </x:c>
+      <x:c r="O99" s="23" t="n">
+        <x:v>15210784</x:v>
+      </x:c>
+      <x:c r="P99" s="23" t="n">
+        <x:v>35122812</x:v>
+      </x:c>
+      <x:c r="Q99" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R99" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S99" s="23" t="n">
+        <x:v>5822000</x:v>
+      </x:c>
+      <x:c r="T99" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U99" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V99" s="25" t="n">
+        <x:f>N99+1.5*O99+3*P99+3*Q99</x:f>
+        <x:v>162347072</x:v>
+      </x:c>
+      <x:c r="W99" s="25" t="n">
+        <x:f>S99*3</x:f>
+        <x:v>17466000</x:v>
+      </x:c>
+      <x:c r="X99" s="25" t="n">
+        <x:f>IF(Z99="No",0,V99-W99)</x:f>
+        <x:v>144881072</x:v>
+      </x:c>
+      <x:c r="Y99" s="26" t="n">
+        <x:f>IF(Z99="No",0,IFERROR(V99/W99,0))</x:f>
+        <x:v>9.295034466964388</x:v>
+      </x:c>
+      <x:c r="Z99" s="27" t="str">
+        <x:f>IF(AND(U99=TRUE,V99=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA99" s="27" t="str">
+        <x:f>IF(Z99="No","Not comparable",IF(X99&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="20" t="str">
+        <x:v>s150-20261002-11</x:v>
+      </x:c>
+      <x:c r="B100" s="21" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C100" s="22" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D100" s="20" t="str">
+        <x:v>PTS scan card</x:v>
+      </x:c>
+      <x:c r="E100" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F100" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G100" s="23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H100" s="23" t="n">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="I100" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J100" s="23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K100" s="23" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="L100" s="23" t="n">
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="M100" s="20" t="str">
+        <x:v>possible</x:v>
+      </x:c>
+      <x:c r="N100" s="23" t="n">
+        <x:v>8367185</x:v>
+      </x:c>
+      <x:c r="O100" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P100" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q100" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R100" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S100" s="23" t="n">
+        <x:v>1393000</x:v>
+      </x:c>
+      <x:c r="T100" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U100" s="24" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V100" s="25" t="n">
+        <x:f>N100+1.5*O100+3*P100+3*Q100</x:f>
+        <x:v>8367185</x:v>
+      </x:c>
+      <x:c r="W100" s="25" t="n">
+        <x:f>S100*3</x:f>
+        <x:v>4179000</x:v>
+      </x:c>
+      <x:c r="X100" s="25" t="n">
+        <x:f>IF(Z100="No",0,V100-W100)</x:f>
+        <x:v>4188185</x:v>
+      </x:c>
+      <x:c r="Y100" s="26" t="n">
+        <x:f>IF(Z100="No",0,IFERROR(V100/W100,0))</x:f>
+        <x:v>2.00219789423307</x:v>
+      </x:c>
+      <x:c r="Z100" s="27" t="str">
+        <x:f>IF(AND(U100=TRUE,V100=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA100" s="27" t="str">
+        <x:f>IF(Z100="No","Not comparable",IF(X100&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="20" t="str">
+        <x:v>delivery-metal-626-pve-4star-collected</x:v>
+      </x:c>
+      <x:c r="B101" s="21" t="n">
+        <x:v>46296</x:v>
+      </x:c>
+      <x:c r="C101" s="22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="D101" s="20" t="str">
+        <x:v>PTS reward claim dialog</x:v>
+      </x:c>
+      <x:c r="E101" s="20" t="str">
+        <x:v>Delivery: Metal</x:v>
+      </x:c>
+      <x:c r="F101" s="20" t="str">
+        <x:v>PvE</x:v>
+      </x:c>
+      <x:c r="G101" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H101" s="23" t="n">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="I101" s="23" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="J101" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K101" s="23" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="L101" s="23" t="n">
+        <x:v>3555</x:v>
+      </x:c>
+      <x:c r="M101" s="20" t="str">
+        <x:v>collected</x:v>
+      </x:c>
+      <x:c r="N101" s="23" t="n">
+        <x:v>59634076</x:v>
+      </x:c>
+      <x:c r="O101" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P101" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q101" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R101" s="24" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S101" s="23" t="n">
+        <x:v>14073696</x:v>
+      </x:c>
+      <x:c r="T101" s="24" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U101" s="24" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V101" s="25" t="n">
+        <x:f>N101+1.5*O101+3*P101+3*Q101</x:f>
+        <x:v>59634076</x:v>
+      </x:c>
+      <x:c r="W101" s="25" t="n">
+        <x:f>S101*3</x:f>
+        <x:v>42221088</x:v>
+      </x:c>
+      <x:c r="X101" s="25" t="n">
+        <x:f>IF(Z101="No",0,V101-W101)</x:f>
+        <x:v>17412988</x:v>
+      </x:c>
+      <x:c r="Y101" s="26" t="n">
+        <x:f>IF(Z101="No",0,IFERROR(V101/W101,0))</x:f>
+        <x:v>1.4124239526939713</x:v>
+      </x:c>
+      <x:c r="Z101" s="27" t="str">
+        <x:f>IF(AND(U101=TRUE,V101=0),"No","Yes")</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AA101" s="27" t="str">
+        <x:f>IF(Z101="No","Not comparable",IF(X101&gt;0,"Yes","No"))</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="X2:X66">
+  <x:conditionalFormatting sqref="X2:X101">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5873c4e6c43c41a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae77b31e3d4c45c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Update guide for Orion beta13 changes
</commit_message>
<xml_diff>
--- a/downloads/orion-mission-research.xlsx
+++ b/downloads/orion-mission-research.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5913374349244e72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mission Data" sheetId="2" r:id="Rb16f065e3be94961"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R4e32b0173d064f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcad77f718d95430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mission Data" sheetId="2" r:id="R56f05c9141084f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R06e59cceca174b75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -78,7 +78,13 @@
     </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -814,8 +820,8 @@
       <x:c r="A2" s="20" t="str">
         <x:v>resource-metal-508-pve-5star-150</x:v>
       </x:c>
-      <x:c r="B2" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B2" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C2" s="22" t="n">
         <x:v>150</x:v>
@@ -906,8 +912,8 @@
       <x:c r="A3" s="20" t="str">
         <x:v>resource-crystal-436-pve-4star-150</x:v>
       </x:c>
-      <x:c r="B3" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B3" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C3" s="22" t="n">
         <x:v>150</x:v>
@@ -998,8 +1004,8 @@
       <x:c r="A4" s="20" t="str">
         <x:v>delivery-metal-595-pvp-2star-150</x:v>
       </x:c>
-      <x:c r="B4" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B4" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C4" s="22" t="n">
         <x:v>150</x:v>
@@ -1090,8 +1096,8 @@
       <x:c r="A5" s="20" t="str">
         <x:v>alien-encounter-490-pve-2star-150</x:v>
       </x:c>
-      <x:c r="B5" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B5" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C5" s="22" t="n">
         <x:v>150</x:v>
@@ -1182,8 +1188,8 @@
       <x:c r="A6" s="20" t="str">
         <x:v>medium-alien-encounter-492-pve-1star-150</x:v>
       </x:c>
-      <x:c r="B6" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B6" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C6" s="22" t="n">
         <x:v>150</x:v>
@@ -1274,8 +1280,8 @@
       <x:c r="A7" s="20" t="str">
         <x:v>lifeform-rescue-404-pve-1star-150</x:v>
       </x:c>
-      <x:c r="B7" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B7" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C7" s="22" t="n">
         <x:v>150</x:v>
@@ -1366,8 +1372,8 @@
       <x:c r="A8" s="20" t="str">
         <x:v>small-alien-encounter-503-pvp-5star-150</x:v>
       </x:c>
-      <x:c r="B8" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B8" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C8" s="22" t="n">
         <x:v>150</x:v>
@@ -1458,8 +1464,8 @@
       <x:c r="A9" s="20" t="str">
         <x:v>chaos-mission-404-pve-5star-150</x:v>
       </x:c>
-      <x:c r="B9" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B9" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C9" s="22" t="n">
         <x:v>150</x:v>
@@ -1550,8 +1556,8 @@
       <x:c r="A10" s="20" t="str">
         <x:v>small-alien-encounter-525-pvp-1star-150</x:v>
       </x:c>
-      <x:c r="B10" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B10" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C10" s="22" t="n">
         <x:v>150</x:v>
@@ -1642,8 +1648,8 @@
       <x:c r="A11" s="20" t="str">
         <x:v>delivery-crystal-471-pvp-1star-150</x:v>
       </x:c>
-      <x:c r="B11" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B11" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C11" s="22" t="n">
         <x:v>150</x:v>
@@ -1734,8 +1740,8 @@
       <x:c r="A12" s="20" t="str">
         <x:v>delivery-crystal-517-pve-4star-150</x:v>
       </x:c>
-      <x:c r="B12" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B12" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C12" s="22" t="n">
         <x:v>150</x:v>
@@ -1826,8 +1832,8 @@
       <x:c r="A13" s="20" t="str">
         <x:v>delivery-metal-502-pvp-3star-150</x:v>
       </x:c>
-      <x:c r="B13" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B13" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C13" s="22" t="n">
         <x:v>150</x:v>
@@ -1918,8 +1924,8 @@
       <x:c r="A14" s="20" t="str">
         <x:v>defend-446-pvp-5star-150</x:v>
       </x:c>
-      <x:c r="B14" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B14" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C14" s="22" t="n">
         <x:v>150</x:v>
@@ -2010,8 +2016,8 @@
       <x:c r="A15" s="20" t="str">
         <x:v>resource-crystal-543-pvp-4star-150</x:v>
       </x:c>
-      <x:c r="B15" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B15" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C15" s="22" t="n">
         <x:v>150</x:v>
@@ -2102,8 +2108,8 @@
       <x:c r="A16" s="20" t="str">
         <x:v>small-alien-encounter-419-pvp-1star-150</x:v>
       </x:c>
-      <x:c r="B16" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B16" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C16" s="22" t="n">
         <x:v>150</x:v>
@@ -2192,8 +2198,8 @@
       <x:c r="A17" s="20" t="str">
         <x:v>small-alien-encounter-557-pve-2star-150</x:v>
       </x:c>
-      <x:c r="B17" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B17" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C17" s="22" t="n">
         <x:v>150</x:v>
@@ -2284,8 +2290,8 @@
       <x:c r="A18" s="20" t="str">
         <x:v>rescue-540-pvp-3star-150</x:v>
       </x:c>
-      <x:c r="B18" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B18" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C18" s="22" t="n">
         <x:v>150</x:v>
@@ -2376,8 +2382,8 @@
       <x:c r="A19" s="20" t="str">
         <x:v>delivery-crystal-505-pve-5star-150</x:v>
       </x:c>
-      <x:c r="B19" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B19" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C19" s="22" t="n">
         <x:v>150</x:v>
@@ -2468,8 +2474,8 @@
       <x:c r="A20" s="20" t="str">
         <x:v>delivery-metal-430-pve-3star-150</x:v>
       </x:c>
-      <x:c r="B20" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B20" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C20" s="22" t="n">
         <x:v>150</x:v>
@@ -2560,8 +2566,8 @@
       <x:c r="A21" s="20" t="str">
         <x:v>lifeform-rescue-564-pve-5star-150</x:v>
       </x:c>
-      <x:c r="B21" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B21" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C21" s="22" t="n">
         <x:v>150</x:v>
@@ -2650,8 +2656,8 @@
       <x:c r="A22" s="20" t="str">
         <x:v>lifeform-rescue-377-pvp-4star-10</x:v>
       </x:c>
-      <x:c r="B22" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B22" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C22" s="22" t="n">
         <x:v>10</x:v>
@@ -2742,8 +2748,8 @@
       <x:c r="A23" s="20" t="str">
         <x:v>delivery-crystal-381-pvp-4star-10</x:v>
       </x:c>
-      <x:c r="B23" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B23" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C23" s="22" t="n">
         <x:v>10</x:v>
@@ -2834,8 +2840,8 @@
       <x:c r="A24" s="20" t="str">
         <x:v>valuable-delivery-430-pvp-1star-10</x:v>
       </x:c>
-      <x:c r="B24" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B24" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C24" s="22" t="n">
         <x:v>10</x:v>
@@ -2926,8 +2932,8 @@
       <x:c r="A25" s="20" t="str">
         <x:v>medium-pirate-encounter-344-pve-4star-50</x:v>
       </x:c>
-      <x:c r="B25" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B25" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C25" s="22" t="n">
         <x:v>50</x:v>
@@ -3018,8 +3024,8 @@
       <x:c r="A26" s="20" t="str">
         <x:v>medium-alien-encounter-410-pve-2star-50</x:v>
       </x:c>
-      <x:c r="B26" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B26" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C26" s="22" t="n">
         <x:v>50</x:v>
@@ -3110,8 +3116,8 @@
       <x:c r="A27" s="20" t="str">
         <x:v>rescue-373-pvp-3star-50</x:v>
       </x:c>
-      <x:c r="B27" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B27" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C27" s="22" t="n">
         <x:v>50</x:v>
@@ -3202,8 +3208,8 @@
       <x:c r="A28" s="20" t="str">
         <x:v>lost-debris-field-384-pve-3star-50</x:v>
       </x:c>
-      <x:c r="B28" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B28" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C28" s="22" t="n">
         <x:v>50</x:v>
@@ -3294,8 +3300,8 @@
       <x:c r="A29" s="20" t="str">
         <x:v>small-alien-encounter-320-pvp-3star-50</x:v>
       </x:c>
-      <x:c r="B29" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B29" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C29" s="22" t="n">
         <x:v>50</x:v>
@@ -3386,8 +3392,8 @@
       <x:c r="A30" s="20" t="str">
         <x:v>delivery-metal-468-pvp-5star-50</x:v>
       </x:c>
-      <x:c r="B30" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B30" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C30" s="22" t="n">
         <x:v>50</x:v>
@@ -3478,8 +3484,8 @@
       <x:c r="A31" s="20" t="str">
         <x:v>rescue-486-pvp-5star</x:v>
       </x:c>
-      <x:c r="B31" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B31" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C31" s="22" t="n">
         <x:v>10</x:v>
@@ -3570,8 +3576,8 @@
       <x:c r="A32" s="20" t="str">
         <x:v>resource-deuterium-578-pve-2star</x:v>
       </x:c>
-      <x:c r="B32" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B32" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C32" s="22" t="n">
         <x:v>10</x:v>
@@ -3662,8 +3668,8 @@
       <x:c r="A33" s="20" t="str">
         <x:v>medium-alien-encounter-673-pvp-3star</x:v>
       </x:c>
-      <x:c r="B33" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B33" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C33" s="22" t="n">
         <x:v>10</x:v>
@@ -3754,8 +3760,8 @@
       <x:c r="A34" s="20" t="str">
         <x:v>delivery-metal-575-pve-3star</x:v>
       </x:c>
-      <x:c r="B34" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B34" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C34" s="22" t="n">
         <x:v>10</x:v>
@@ -3846,8 +3852,8 @@
       <x:c r="A35" s="20" t="str">
         <x:v>rescue-692-pvp-2star</x:v>
       </x:c>
-      <x:c r="B35" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B35" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C35" s="22" t="n">
         <x:v>10</x:v>
@@ -3938,8 +3944,8 @@
       <x:c r="A36" s="20" t="str">
         <x:v>delivery-crystal-568-pve-3star</x:v>
       </x:c>
-      <x:c r="B36" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B36" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C36" s="22" t="n">
         <x:v>10</x:v>
@@ -4030,8 +4036,8 @@
       <x:c r="A37" s="20" t="str">
         <x:v>medium-pirate-encounter-585-pve-3star</x:v>
       </x:c>
-      <x:c r="B37" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B37" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C37" s="22" t="n">
         <x:v>10</x:v>
@@ -4122,8 +4128,8 @@
       <x:c r="A38" s="20" t="str">
         <x:v>small-alien-encounter-629-pvp-1star</x:v>
       </x:c>
-      <x:c r="B38" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B38" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C38" s="22" t="n">
         <x:v>10</x:v>
@@ -4214,8 +4220,8 @@
       <x:c r="A39" s="20" t="str">
         <x:v>medium-alien-encounter-478-pve-4star</x:v>
       </x:c>
-      <x:c r="B39" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B39" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C39" s="22" t="n">
         <x:v>10</x:v>
@@ -4306,8 +4312,8 @@
       <x:c r="A40" s="20" t="str">
         <x:v>delivery-metal-522-pve-4star</x:v>
       </x:c>
-      <x:c r="B40" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B40" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C40" s="22" t="n">
         <x:v>10</x:v>
@@ -4398,8 +4404,8 @@
       <x:c r="A41" s="20" t="str">
         <x:v>resource-metal-698-pvp-3star</x:v>
       </x:c>
-      <x:c r="B41" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B41" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C41" s="22" t="n">
         <x:v>10</x:v>
@@ -4490,8 +4496,8 @@
       <x:c r="A42" s="20" t="str">
         <x:v>delivery-metal-628-pvp-1star</x:v>
       </x:c>
-      <x:c r="B42" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B42" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C42" s="22" t="n">
         <x:v>10</x:v>
@@ -4582,8 +4588,8 @@
       <x:c r="A43" s="20" t="str">
         <x:v>delivery-metal-685-pve-2star</x:v>
       </x:c>
-      <x:c r="B43" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B43" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C43" s="22" t="n">
         <x:v>10</x:v>
@@ -4674,8 +4680,8 @@
       <x:c r="A44" s="20" t="str">
         <x:v>delivery-crystal-535-pvp-2star</x:v>
       </x:c>
-      <x:c r="B44" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B44" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C44" s="22" t="n">
         <x:v>10</x:v>
@@ -4766,8 +4772,8 @@
       <x:c r="A45" s="20" t="str">
         <x:v>delivery-deuterium-577-pve-1star</x:v>
       </x:c>
-      <x:c r="B45" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B45" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C45" s="22" t="n">
         <x:v>10</x:v>
@@ -4858,8 +4864,8 @@
       <x:c r="A46" s="20" t="str">
         <x:v>small-alien-encounter-643-pve-1star</x:v>
       </x:c>
-      <x:c r="B46" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B46" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C46" s="22" t="n">
         <x:v>10</x:v>
@@ -4950,8 +4956,8 @@
       <x:c r="A47" s="20" t="str">
         <x:v>alien-encounter-534-pvp-1star</x:v>
       </x:c>
-      <x:c r="B47" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B47" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C47" s="22" t="n">
         <x:v>50</x:v>
@@ -5042,8 +5048,8 @@
       <x:c r="A48" s="20" t="str">
         <x:v>rescue-706-pve-5star</x:v>
       </x:c>
-      <x:c r="B48" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B48" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C48" s="22" t="n">
         <x:v>50</x:v>
@@ -5132,8 +5138,8 @@
       <x:c r="A49" s="20" t="str">
         <x:v>medium-alien-encounter-610-pve-1star</x:v>
       </x:c>
-      <x:c r="B49" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B49" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C49" s="22" t="n">
         <x:v>50</x:v>
@@ -5224,8 +5230,8 @@
       <x:c r="A50" s="20" t="str">
         <x:v>medium-alien-encounter-690-pvp-3star</x:v>
       </x:c>
-      <x:c r="B50" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B50" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C50" s="22" t="n">
         <x:v>50</x:v>
@@ -5316,8 +5322,8 @@
       <x:c r="A51" s="20" t="str">
         <x:v>delivery-crystal-640-pve-2star</x:v>
       </x:c>
-      <x:c r="B51" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B51" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C51" s="22" t="n">
         <x:v>50</x:v>
@@ -5408,8 +5414,8 @@
       <x:c r="A52" s="20" t="str">
         <x:v>medium-pirate-encounter-581-pve-3star</x:v>
       </x:c>
-      <x:c r="B52" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B52" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C52" s="22" t="n">
         <x:v>50</x:v>
@@ -5498,8 +5504,8 @@
       <x:c r="A53" s="20" t="str">
         <x:v>delivery-metal-708-pvp-4star</x:v>
       </x:c>
-      <x:c r="B53" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B53" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C53" s="22" t="n">
         <x:v>50</x:v>
@@ -5590,8 +5596,8 @@
       <x:c r="A54" s="20" t="str">
         <x:v>small-alien-encounter-527-pvp-2star</x:v>
       </x:c>
-      <x:c r="B54" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B54" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C54" s="22" t="n">
         <x:v>50</x:v>
@@ -5682,8 +5688,8 @@
       <x:c r="A55" s="20" t="str">
         <x:v>alien-encounter-619-pve-1star</x:v>
       </x:c>
-      <x:c r="B55" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B55" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C55" s="22" t="n">
         <x:v>50</x:v>
@@ -5774,8 +5780,8 @@
       <x:c r="A56" s="20" t="str">
         <x:v>delivery-crystal-549-pvp-2star</x:v>
       </x:c>
-      <x:c r="B56" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B56" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C56" s="22" t="n">
         <x:v>50</x:v>
@@ -5866,8 +5872,8 @@
       <x:c r="A57" s="20" t="str">
         <x:v>defend-658-pvp-2star</x:v>
       </x:c>
-      <x:c r="B57" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B57" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C57" s="22" t="n">
         <x:v>50</x:v>
@@ -5956,8 +5962,8 @@
       <x:c r="A58" s="20" t="str">
         <x:v>small-alien-encounter-501-pve-5star</x:v>
       </x:c>
-      <x:c r="B58" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B58" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C58" s="22" t="n">
         <x:v>50</x:v>
@@ -6048,8 +6054,8 @@
       <x:c r="A59" s="20" t="str">
         <x:v>chaos-mission-669-pve-4star</x:v>
       </x:c>
-      <x:c r="B59" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B59" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C59" s="22" t="n">
         <x:v>150</x:v>
@@ -6140,8 +6146,8 @@
       <x:c r="A60" s="20" t="str">
         <x:v>medium-pirate-encounter-542-pvp-1star</x:v>
       </x:c>
-      <x:c r="B60" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B60" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C60" s="22" t="n">
         <x:v>150</x:v>
@@ -6232,8 +6238,8 @@
       <x:c r="A61" s="20" t="str">
         <x:v>medium-alien-encounter-490-pve-4star</x:v>
       </x:c>
-      <x:c r="B61" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B61" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C61" s="22" t="n">
         <x:v>150</x:v>
@@ -6324,8 +6330,8 @@
       <x:c r="A62" s="20" t="str">
         <x:v>small-alien-encounter-620-pve-1star</x:v>
       </x:c>
-      <x:c r="B62" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B62" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C62" s="22" t="n">
         <x:v>150</x:v>
@@ -6416,8 +6422,8 @@
       <x:c r="A63" s="20" t="str">
         <x:v>valuable-delivery-486-pvp-1star</x:v>
       </x:c>
-      <x:c r="B63" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B63" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C63" s="22" t="n">
         <x:v>150</x:v>
@@ -6508,8 +6514,8 @@
       <x:c r="A64" s="20" t="str">
         <x:v>mysterious-nebula-499-pvp-1star</x:v>
       </x:c>
-      <x:c r="B64" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B64" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C64" s="22" t="n">
         <x:v>150</x:v>
@@ -6600,8 +6606,8 @@
       <x:c r="A65" s="20" t="str">
         <x:v>medium-alien-encounter-617-pve-1star</x:v>
       </x:c>
-      <x:c r="B65" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B65" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C65" s="22" t="n">
         <x:v>150</x:v>
@@ -6692,8 +6698,8 @@
       <x:c r="A66" s="20" t="str">
         <x:v>small-alien-encounter-655-pvp-4star</x:v>
       </x:c>
-      <x:c r="B66" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B66" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C66" s="22" t="n">
         <x:v>150</x:v>
@@ -6784,8 +6790,8 @@
       <x:c r="A67" s="20" t="str">
         <x:v>small-alien-encounter-534-pve-3star</x:v>
       </x:c>
-      <x:c r="B67" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B67" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C67" s="22" t="n">
         <x:v>150</x:v>
@@ -6876,8 +6882,8 @@
       <x:c r="A68" s="20" t="str">
         <x:v>lost-debris-field-527-pvp-5star</x:v>
       </x:c>
-      <x:c r="B68" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B68" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C68" s="22" t="n">
         <x:v>150</x:v>
@@ -6968,8 +6974,8 @@
       <x:c r="A69" s="20" t="str">
         <x:v>valuable-delivery-619-pvp-1star</x:v>
       </x:c>
-      <x:c r="B69" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B69" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C69" s="22" t="n">
         <x:v>150</x:v>
@@ -7060,8 +7066,8 @@
       <x:c r="A70" s="20" t="str">
         <x:v>delivery-crystal-513-pve-2star</x:v>
       </x:c>
-      <x:c r="B70" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B70" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C70" s="22" t="n">
         <x:v>150</x:v>
@@ -7152,8 +7158,8 @@
       <x:c r="A71" s="20" t="str">
         <x:v>medium-alien-encounter-373-pvp-1star</x:v>
       </x:c>
-      <x:c r="B71" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B71" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C71" s="22" t="n">
         <x:v>10</x:v>
@@ -7244,8 +7250,8 @@
       <x:c r="A72" s="20" t="str">
         <x:v>small-alien-encounter-277-pvp-5star</x:v>
       </x:c>
-      <x:c r="B72" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B72" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C72" s="22" t="n">
         <x:v>10</x:v>
@@ -7336,8 +7342,8 @@
       <x:c r="A73" s="20" t="str">
         <x:v>resource-deuterium-370-pve-1star</x:v>
       </x:c>
-      <x:c r="B73" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B73" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C73" s="22" t="n">
         <x:v>10</x:v>
@@ -7428,8 +7434,8 @@
       <x:c r="A74" s="20" t="str">
         <x:v>resource-metal-358-pvp-4star</x:v>
       </x:c>
-      <x:c r="B74" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B74" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C74" s="22" t="n">
         <x:v>10</x:v>
@@ -7520,8 +7526,8 @@
       <x:c r="A75" s="20" t="str">
         <x:v>delivery-crystal-280-pvp-4star</x:v>
       </x:c>
-      <x:c r="B75" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B75" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C75" s="22" t="n">
         <x:v>50</x:v>
@@ -7612,8 +7618,8 @@
       <x:c r="A76" s="20" t="str">
         <x:v>small-alien-encounter-359-pve-2star</x:v>
       </x:c>
-      <x:c r="B76" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B76" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C76" s="22" t="n">
         <x:v>50</x:v>
@@ -7704,8 +7710,8 @@
       <x:c r="A77" s="20" t="str">
         <x:v>resource-crystal-340-pve-1star</x:v>
       </x:c>
-      <x:c r="B77" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B77" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C77" s="22" t="n">
         <x:v>50</x:v>
@@ -7796,8 +7802,8 @@
       <x:c r="A78" s="20" t="str">
         <x:v>delivery-deuterium-316-pve-2star</x:v>
       </x:c>
-      <x:c r="B78" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B78" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C78" s="22" t="n">
         <x:v>50</x:v>
@@ -7888,8 +7894,8 @@
       <x:c r="A79" s="20" t="str">
         <x:v>delivery-metal-280-pve-1star</x:v>
       </x:c>
-      <x:c r="B79" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B79" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C79" s="22" t="n">
         <x:v>150</x:v>
@@ -7980,8 +7986,8 @@
       <x:c r="A80" s="20" t="str">
         <x:v>medium-alien-encounter-383-pve-5star</x:v>
       </x:c>
-      <x:c r="B80" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B80" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C80" s="22" t="n">
         <x:v>150</x:v>
@@ -8072,8 +8078,8 @@
       <x:c r="A81" s="20" t="str">
         <x:v>medium-alien-encounter-297-pve-1star</x:v>
       </x:c>
-      <x:c r="B81" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B81" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C81" s="22" t="n">
         <x:v>150</x:v>
@@ -8164,8 +8170,8 @@
       <x:c r="A82" s="20" t="str">
         <x:v>alien-encounter-259-pvp-5star</x:v>
       </x:c>
-      <x:c r="B82" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B82" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C82" s="22" t="n">
         <x:v>150</x:v>
@@ -8256,8 +8262,8 @@
       <x:c r="A83" s="20" t="str">
         <x:v>resource-metal-462-pve-1star</x:v>
       </x:c>
-      <x:c r="B83" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B83" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C83" s="22" t="n">
         <x:v>10</x:v>
@@ -8348,8 +8354,8 @@
       <x:c r="A84" s="20" t="str">
         <x:v>delivery-crystal-521-pve-2star</x:v>
       </x:c>
-      <x:c r="B84" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B84" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C84" s="22" t="n">
         <x:v>10</x:v>
@@ -8440,8 +8446,8 @@
       <x:c r="A85" s="20" t="str">
         <x:v>rescue-408-pve-2star</x:v>
       </x:c>
-      <x:c r="B85" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B85" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C85" s="22" t="n">
         <x:v>10</x:v>
@@ -8530,8 +8536,8 @@
       <x:c r="A86" s="20" t="str">
         <x:v>alien-encounter-514-pve-1star</x:v>
       </x:c>
-      <x:c r="B86" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B86" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C86" s="22" t="n">
         <x:v>10</x:v>
@@ -8622,8 +8628,8 @@
       <x:c r="A87" s="20" t="str">
         <x:v>small-alien-encounter-443-pve-1star</x:v>
       </x:c>
-      <x:c r="B87" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B87" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C87" s="22" t="n">
         <x:v>50</x:v>
@@ -8712,8 +8718,8 @@
       <x:c r="A88" s="20" t="str">
         <x:v>defend-480-pve-4star</x:v>
       </x:c>
-      <x:c r="B88" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B88" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C88" s="22" t="n">
         <x:v>50</x:v>
@@ -8802,8 +8808,8 @@
       <x:c r="A89" s="20" t="str">
         <x:v>delivery-metal-409-pvp-4star</x:v>
       </x:c>
-      <x:c r="B89" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B89" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C89" s="22" t="n">
         <x:v>50</x:v>
@@ -8894,8 +8900,8 @@
       <x:c r="A90" s="20" t="str">
         <x:v>medium-alien-encounter-452-pve-1star</x:v>
       </x:c>
-      <x:c r="B90" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B90" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C90" s="22" t="n">
         <x:v>50</x:v>
@@ -8986,8 +8992,8 @@
       <x:c r="A91" s="20" t="str">
         <x:v>mysterious-nebula-411-pve-3star</x:v>
       </x:c>
-      <x:c r="B91" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B91" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C91" s="22" t="n">
         <x:v>150</x:v>
@@ -9076,8 +9082,8 @@
       <x:c r="A92" s="20" t="str">
         <x:v>small-alien-encounter-506-pvp-3star</x:v>
       </x:c>
-      <x:c r="B92" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B92" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C92" s="22" t="n">
         <x:v>150</x:v>
@@ -9168,8 +9174,8 @@
       <x:c r="A93" s="20" t="str">
         <x:v>medium-pirate-encounter-409-pve-4star</x:v>
       </x:c>
-      <x:c r="B93" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B93" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C93" s="22" t="n">
         <x:v>150</x:v>
@@ -9260,8 +9266,8 @@
       <x:c r="A94" s="20" t="str">
         <x:v>rescue-413-pve-1star</x:v>
       </x:c>
-      <x:c r="B94" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B94" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C94" s="22" t="n">
         <x:v>150</x:v>
@@ -9352,8 +9358,8 @@
       <x:c r="A95" s="20" t="str">
         <x:v>s10-20261002-01</x:v>
       </x:c>
-      <x:c r="B95" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B95" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C95" s="22" t="n">
         <x:v>10</x:v>
@@ -9444,8 +9450,8 @@
       <x:c r="A96" s="20" t="str">
         <x:v>s10-20261002-02</x:v>
       </x:c>
-      <x:c r="B96" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B96" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C96" s="22" t="n">
         <x:v>10</x:v>
@@ -9536,8 +9542,8 @@
       <x:c r="A97" s="20" t="str">
         <x:v>s10-20261002-03</x:v>
       </x:c>
-      <x:c r="B97" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B97" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C97" s="22" t="n">
         <x:v>10</x:v>
@@ -9626,8 +9632,8 @@
       <x:c r="A98" s="20" t="str">
         <x:v>s10-20261002-04</x:v>
       </x:c>
-      <x:c r="B98" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B98" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C98" s="22" t="n">
         <x:v>10</x:v>
@@ -9718,8 +9724,8 @@
       <x:c r="A99" s="20" t="str">
         <x:v>s10-20261002-05</x:v>
       </x:c>
-      <x:c r="B99" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B99" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C99" s="22" t="n">
         <x:v>10</x:v>
@@ -9810,8 +9816,8 @@
       <x:c r="A100" s="20" t="str">
         <x:v>s10-20261002-06</x:v>
       </x:c>
-      <x:c r="B100" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B100" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C100" s="22" t="n">
         <x:v>10</x:v>
@@ -9902,8 +9908,8 @@
       <x:c r="A101" s="20" t="str">
         <x:v>s10-20261002-07</x:v>
       </x:c>
-      <x:c r="B101" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B101" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C101" s="22" t="n">
         <x:v>10</x:v>
@@ -9994,8 +10000,8 @@
       <x:c r="A102" s="20" t="str">
         <x:v>s10-20261002-08</x:v>
       </x:c>
-      <x:c r="B102" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B102" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C102" s="22" t="n">
         <x:v>10</x:v>
@@ -10086,8 +10092,8 @@
       <x:c r="A103" s="20" t="str">
         <x:v>s10-20261002-09</x:v>
       </x:c>
-      <x:c r="B103" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B103" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C103" s="22" t="n">
         <x:v>10</x:v>
@@ -10178,8 +10184,8 @@
       <x:c r="A104" s="20" t="str">
         <x:v>s10-20261002-10</x:v>
       </x:c>
-      <x:c r="B104" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B104" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C104" s="22" t="n">
         <x:v>10</x:v>
@@ -10270,8 +10276,8 @@
       <x:c r="A105" s="20" t="str">
         <x:v>s10-20261002-11</x:v>
       </x:c>
-      <x:c r="B105" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B105" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C105" s="22" t="n">
         <x:v>10</x:v>
@@ -10362,8 +10368,8 @@
       <x:c r="A106" s="20" t="str">
         <x:v>s10-20261002-12</x:v>
       </x:c>
-      <x:c r="B106" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B106" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C106" s="22" t="n">
         <x:v>10</x:v>
@@ -10454,8 +10460,8 @@
       <x:c r="A107" s="20" t="str">
         <x:v>s50-20261002-01</x:v>
       </x:c>
-      <x:c r="B107" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B107" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C107" s="22" t="n">
         <x:v>50</x:v>
@@ -10546,8 +10552,8 @@
       <x:c r="A108" s="20" t="str">
         <x:v>s50-20261002-02</x:v>
       </x:c>
-      <x:c r="B108" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B108" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C108" s="22" t="n">
         <x:v>50</x:v>
@@ -10638,8 +10644,8 @@
       <x:c r="A109" s="20" t="str">
         <x:v>s50-20261002-03</x:v>
       </x:c>
-      <x:c r="B109" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B109" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C109" s="22" t="n">
         <x:v>50</x:v>
@@ -10728,8 +10734,8 @@
       <x:c r="A110" s="20" t="str">
         <x:v>s50-20261002-04</x:v>
       </x:c>
-      <x:c r="B110" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B110" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C110" s="22" t="n">
         <x:v>50</x:v>
@@ -10820,8 +10826,8 @@
       <x:c r="A111" s="20" t="str">
         <x:v>s50-20261002-05</x:v>
       </x:c>
-      <x:c r="B111" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B111" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C111" s="22" t="n">
         <x:v>50</x:v>
@@ -10912,8 +10918,8 @@
       <x:c r="A112" s="20" t="str">
         <x:v>s50-20261002-06</x:v>
       </x:c>
-      <x:c r="B112" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B112" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C112" s="22" t="n">
         <x:v>50</x:v>
@@ -11004,8 +11010,8 @@
       <x:c r="A113" s="20" t="str">
         <x:v>s50-20261002-07</x:v>
       </x:c>
-      <x:c r="B113" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B113" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C113" s="22" t="n">
         <x:v>50</x:v>
@@ -11096,8 +11102,8 @@
       <x:c r="A114" s="20" t="str">
         <x:v>s50-20261002-08</x:v>
       </x:c>
-      <x:c r="B114" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B114" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C114" s="22" t="n">
         <x:v>50</x:v>
@@ -11188,8 +11194,8 @@
       <x:c r="A115" s="20" t="str">
         <x:v>s50-20261002-09</x:v>
       </x:c>
-      <x:c r="B115" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B115" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C115" s="22" t="n">
         <x:v>50</x:v>
@@ -11280,8 +11286,8 @@
       <x:c r="A116" s="20" t="str">
         <x:v>s50-20261002-10</x:v>
       </x:c>
-      <x:c r="B116" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B116" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C116" s="22" t="n">
         <x:v>50</x:v>
@@ -11372,8 +11378,8 @@
       <x:c r="A117" s="20" t="str">
         <x:v>s50-20261002-11</x:v>
       </x:c>
-      <x:c r="B117" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B117" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C117" s="22" t="n">
         <x:v>50</x:v>
@@ -11464,8 +11470,8 @@
       <x:c r="A118" s="20" t="str">
         <x:v>s50-20261002-12</x:v>
       </x:c>
-      <x:c r="B118" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B118" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C118" s="22" t="n">
         <x:v>50</x:v>
@@ -11556,8 +11562,8 @@
       <x:c r="A119" s="20" t="str">
         <x:v>s150-20261002-01</x:v>
       </x:c>
-      <x:c r="B119" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B119" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C119" s="22" t="n">
         <x:v>150</x:v>
@@ -11648,8 +11654,8 @@
       <x:c r="A120" s="20" t="str">
         <x:v>s150-20261002-02</x:v>
       </x:c>
-      <x:c r="B120" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B120" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C120" s="22" t="n">
         <x:v>150</x:v>
@@ -11738,8 +11744,8 @@
       <x:c r="A121" s="20" t="str">
         <x:v>s150-20261002-03</x:v>
       </x:c>
-      <x:c r="B121" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B121" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C121" s="22" t="n">
         <x:v>150</x:v>
@@ -11830,8 +11836,8 @@
       <x:c r="A122" s="20" t="str">
         <x:v>s150-20261002-04</x:v>
       </x:c>
-      <x:c r="B122" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B122" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C122" s="22" t="n">
         <x:v>150</x:v>
@@ -11922,8 +11928,8 @@
       <x:c r="A123" s="20" t="str">
         <x:v>s150-20261002-05</x:v>
       </x:c>
-      <x:c r="B123" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B123" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C123" s="22" t="n">
         <x:v>150</x:v>
@@ -12014,8 +12020,8 @@
       <x:c r="A124" s="20" t="str">
         <x:v>s150-20261002-06</x:v>
       </x:c>
-      <x:c r="B124" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B124" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C124" s="22" t="n">
         <x:v>150</x:v>
@@ -12106,8 +12112,8 @@
       <x:c r="A125" s="20" t="str">
         <x:v>s150-20261002-07</x:v>
       </x:c>
-      <x:c r="B125" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B125" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C125" s="22" t="n">
         <x:v>150</x:v>
@@ -12198,8 +12204,8 @@
       <x:c r="A126" s="20" t="str">
         <x:v>s150-20261002-08</x:v>
       </x:c>
-      <x:c r="B126" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B126" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C126" s="22" t="n">
         <x:v>150</x:v>
@@ -12288,8 +12294,8 @@
       <x:c r="A127" s="20" t="str">
         <x:v>s150-20261002-09</x:v>
       </x:c>
-      <x:c r="B127" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B127" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C127" s="22" t="n">
         <x:v>150</x:v>
@@ -12380,8 +12386,8 @@
       <x:c r="A128" s="20" t="str">
         <x:v>s150-20261002-10</x:v>
       </x:c>
-      <x:c r="B128" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B128" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C128" s="22" t="n">
         <x:v>150</x:v>
@@ -12472,8 +12478,8 @@
       <x:c r="A129" s="20" t="str">
         <x:v>s150-20261002-11</x:v>
       </x:c>
-      <x:c r="B129" s="21" t="n">
-        <x:v>46297</x:v>
+      <x:c r="B129" s="21" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C129" s="22" t="n">
         <x:v>150</x:v>
@@ -12564,8 +12570,8 @@
       <x:c r="A130" s="20" t="str">
         <x:v>delivery-metal-626-pve-4star-collected</x:v>
       </x:c>
-      <x:c r="B130" s="21" t="n">
-        <x:v>46296</x:v>
+      <x:c r="B130" s="21" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C130" s="22" t="str">
         <x:v>Unknown</x:v>
@@ -12656,8 +12662,8 @@
       <x:c r="A131" s="20" t="str">
         <x:v>s150-20261003-01</x:v>
       </x:c>
-      <x:c r="B131" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B131" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C131" s="22" t="n">
         <x:v>150</x:v>
@@ -12748,8 +12754,8 @@
       <x:c r="A132" s="20" t="str">
         <x:v>s150-20261003-02</x:v>
       </x:c>
-      <x:c r="B132" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B132" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C132" s="22" t="n">
         <x:v>150</x:v>
@@ -12840,8 +12846,8 @@
       <x:c r="A133" s="20" t="str">
         <x:v>s150-20261003-03</x:v>
       </x:c>
-      <x:c r="B133" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B133" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C133" s="22" t="n">
         <x:v>150</x:v>
@@ -12932,8 +12938,8 @@
       <x:c r="A134" s="20" t="str">
         <x:v>s150-20261003-04</x:v>
       </x:c>
-      <x:c r="B134" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B134" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C134" s="22" t="n">
         <x:v>150</x:v>
@@ -13024,8 +13030,8 @@
       <x:c r="A135" s="20" t="str">
         <x:v>s150-20261003-05</x:v>
       </x:c>
-      <x:c r="B135" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B135" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C135" s="22" t="n">
         <x:v>150</x:v>
@@ -13116,8 +13122,8 @@
       <x:c r="A136" s="20" t="str">
         <x:v>s150-20261003-06</x:v>
       </x:c>
-      <x:c r="B136" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B136" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C136" s="22" t="n">
         <x:v>150</x:v>
@@ -13208,8 +13214,8 @@
       <x:c r="A137" s="20" t="str">
         <x:v>s150-20261003-07</x:v>
       </x:c>
-      <x:c r="B137" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B137" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C137" s="22" t="n">
         <x:v>150</x:v>
@@ -13298,8 +13304,8 @@
       <x:c r="A138" s="20" t="str">
         <x:v>s150-20261003-08</x:v>
       </x:c>
-      <x:c r="B138" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B138" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C138" s="22" t="n">
         <x:v>150</x:v>
@@ -13390,8 +13396,8 @@
       <x:c r="A139" s="20" t="str">
         <x:v>s150-20261003-09</x:v>
       </x:c>
-      <x:c r="B139" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B139" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C139" s="22" t="n">
         <x:v>150</x:v>
@@ -13482,8 +13488,8 @@
       <x:c r="A140" s="20" t="str">
         <x:v>s150-20261003-10</x:v>
       </x:c>
-      <x:c r="B140" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B140" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C140" s="22" t="n">
         <x:v>150</x:v>
@@ -13574,8 +13580,8 @@
       <x:c r="A141" s="20" t="str">
         <x:v>s150-20261003-11</x:v>
       </x:c>
-      <x:c r="B141" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B141" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C141" s="22" t="n">
         <x:v>150</x:v>
@@ -13666,8 +13672,8 @@
       <x:c r="A142" s="20" t="str">
         <x:v>s150-20261003-12</x:v>
       </x:c>
-      <x:c r="B142" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B142" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C142" s="22" t="n">
         <x:v>150</x:v>
@@ -13758,8 +13764,8 @@
       <x:c r="A143" s="20" t="str">
         <x:v>s150-20261003-13</x:v>
       </x:c>
-      <x:c r="B143" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B143" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C143" s="22" t="n">
         <x:v>150</x:v>
@@ -13848,8 +13854,8 @@
       <x:c r="A144" s="20" t="str">
         <x:v>s150-20261003-14</x:v>
       </x:c>
-      <x:c r="B144" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B144" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C144" s="22" t="n">
         <x:v>150</x:v>
@@ -13935,8 +13941,8 @@
       <x:c r="A145" s="20" t="str">
         <x:v>s150-20261003-15</x:v>
       </x:c>
-      <x:c r="B145" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B145" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C145" s="22" t="n">
         <x:v>150</x:v>
@@ -14027,8 +14033,8 @@
       <x:c r="A146" s="20" t="str">
         <x:v>s150-20261003-16</x:v>
       </x:c>
-      <x:c r="B146" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B146" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C146" s="22" t="n">
         <x:v>150</x:v>
@@ -14119,8 +14125,8 @@
       <x:c r="A147" s="20" t="str">
         <x:v>s150-20261003-17</x:v>
       </x:c>
-      <x:c r="B147" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B147" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C147" s="22" t="n">
         <x:v>150</x:v>
@@ -14209,8 +14215,8 @@
       <x:c r="A148" s="20" t="str">
         <x:v>s150-20261003-18</x:v>
       </x:c>
-      <x:c r="B148" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B148" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C148" s="22" t="n">
         <x:v>150</x:v>
@@ -14301,8 +14307,8 @@
       <x:c r="A149" s="20" t="str">
         <x:v>s150-20261003-19</x:v>
       </x:c>
-      <x:c r="B149" s="21" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B149" s="21" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C149" s="22" t="n">
         <x:v>150</x:v>
@@ -14397,7 +14403,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a5edcc2e871417e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2680f81adfa440e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>